<commit_message>
CBD catalog: add categories, exhibition brief, search, pinyin
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,20 +449,25 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Comment 1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Comment 2</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Comment 3</t>
         </is>
@@ -499,20 +504,25 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>50.000¥. Moq-1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>50.000¥. Moq-1</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>50.000¥. Moq-1</t>
         </is>
@@ -529,20 +539,25 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>500 pcs price 58 usd</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>1000 pcs price 120 usd</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>1000 pcs price 38 USD</t>
         </is>
@@ -579,20 +594,25 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>80$</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>70$</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>300 yuan</t>
         </is>
@@ -629,20 +649,25 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>500pcs / $100USD for pcs</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>50pcs / $50USD for pcs</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>20pcs / $100USD for pcs</t>
         </is>
@@ -675,20 +700,25 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>Custom order</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Custom order</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Custom order</t>
         </is>
@@ -725,20 +755,25 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>170 to 335 usd</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>100 to up</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>100 to up usd</t>
         </is>
@@ -755,20 +790,25 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>Super</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Super</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Super</t>
         </is>
@@ -801,20 +841,25 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>50</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -847,20 +892,25 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>Wall sheet , 200 rmb per meter , 2000 mtr,</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Handles , 500 moq , 100 rmb per handle</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Wall sheet and wooden wall sheet , 2000mtr , 150 rmb per mtr</t>
         </is>
@@ -897,20 +947,25 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>Price: 800 – 2600 CNY per unit depending on the model and features. MOQ: 100 uni</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Price: 1200 – 3500 CNY per unit depending on materials and security specificatio</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Price: 1800 – 4500 CNY per unit based on the finish and decorative complexity. M</t>
         </is>
@@ -943,20 +998,25 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>Хорошее, 400rmb</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Хорошее , 1500rmb</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Нормальное</t>
         </is>
@@ -977,20 +1037,25 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>$176, MOQ 50, very good!</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>$55, MOQ100pcs, good</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>$30, MOQ 10pcs, nice</t>
         </is>
@@ -1027,20 +1092,25 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>1000 yuan 1 square</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>150 rmb</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>570 rmb</t>
         </is>
@@ -1077,20 +1147,25 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>620 super</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>1500 super</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>130 super</t>
         </is>
@@ -1127,20 +1202,25 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>$32, MOQ 300, good</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>¥3000, MoQ 1pcs, very good</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>¥17, Moq 50, good</t>
         </is>
@@ -1177,20 +1257,25 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>600 RMB Great, very cheap</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>800 rmb, little high</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>3400, Good price</t>
         </is>
@@ -1219,20 +1304,25 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>10$</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>69$</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>50-85$</t>
         </is>
@@ -1261,20 +1351,25 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>￥1000 good</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>¥ 500 good</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>￥ 300 good</t>
         </is>
@@ -1303,20 +1398,25 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>300 rmb and more. Good quality and good price. Small quantity</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>33$ for 1 pcs. Good quality and quantity</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Good quality and quantity. 140 rmb 1 pcs.</t>
         </is>
@@ -1341,20 +1441,25 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>Good 👍</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>1570</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
@@ -1391,20 +1496,25 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>130 yuan</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>20000usd</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>500yuan</t>
         </is>
@@ -1441,20 +1551,25 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>MOQ 100, 47 rnb per piece</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>MOQ 50, 200 rnb per</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>MOQ 10, 845 per piece</t>
         </is>
@@ -1491,20 +1606,25 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>1pcs. Start from 60rmb. Novative technology</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>From 1pc. Natural materials.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>1250rmb. MOQ 1 pc</t>
         </is>
@@ -1541,20 +1661,25 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>399</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>199</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>1410</t>
         </is>
@@ -1591,20 +1716,25 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>329</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>229</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>680</t>
         </is>
@@ -1641,20 +1771,25 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>150 yuan, 100, good range of products</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>800usd, very nice, good quality product</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Set of furniture is very good quality, I like the company has also a showroom in</t>
         </is>
@@ -1675,20 +1810,25 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>The price starts from three thousand yuan, the consultant showed all the functio</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>The price starts from three thousand yuan, the consultant showed all the functio</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>I couldn't tell you the price for smart pens right away, but they said they woul</t>
         </is>
@@ -1721,20 +1861,25 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
           <t>199</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>1410</t>
         </is>
@@ -1767,20 +1912,25 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не р</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с е</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно за</t>
         </is>
@@ -1817,20 +1967,25 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного </t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количест</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккур</t>
         </is>
@@ -1867,20 +2022,25 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>2900 usd</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1917,20 +2077,25 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product a</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>MOQ 1, they got samples. 8000usd. Very well made product, trendy and popular. Th</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable</t>
         </is>
@@ -1967,20 +2132,25 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
           <t>600</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>43</t>
         </is>
@@ -2017,20 +2187,25 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
           <t>0.6 usd/m2</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>Under negotiation, great opportunities</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>1-5 usd/l</t>
         </is>
@@ -2063,20 +2238,25 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
           <t>100</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>679 rmb</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>59 rmb</t>
         </is>
@@ -2101,20 +2281,25 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
           <t>249RMB</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>6000RMB</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>2000RMB&amp;gt;</t>
         </is>
@@ -2147,20 +2332,25 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
           <t>MOQ - 5000 and price - 7000 dollars</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>4000$</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>3000 dollars</t>
         </is>
@@ -2193,20 +2383,25 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
           <t>The price cheap, merchant very friendly</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>The price more cheaper, good quality</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Good merchant, perfect products</t>
         </is>
@@ -2243,20 +2438,25 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
           <t>160 RMB/ pcs The prices are attractive and he wants me to represent their produc</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>15 RMB the product is interesting</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>nearly $15,000 for this production line</t>
         </is>
@@ -2293,20 +2493,25 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
           <t>149</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>249</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>749</t>
         </is>
@@ -2343,20 +2548,25 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
           <t>5000 USD</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>3000 USD</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>3000 USD</t>
         </is>
@@ -2381,20 +2591,25 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
           <t>6000 RMB. I like the way they explain everything about their product.</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Smart home system 2000 RMB. They have showed us how the smart home system works.</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>249 RMB. They have fully described their products.</t>
         </is>
@@ -2423,20 +2638,25 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
           <t>6000RMB，积极，详细地告诉了一切</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>249RMB , 价格很便宜</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>2000 RMB</t>
         </is>
@@ -2469,20 +2689,25 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
           <t>400rmb /m2 good meeting</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>350 rmb/m2</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>MOQ 5000 pieces</t>
         </is>
@@ -2515,20 +2740,25 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
           <t>400rmb/m2</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>350rmb/m2</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>MOQ 5000 pieces</t>
         </is>
@@ -2565,20 +2795,25 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
           <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>3000 / MOQ 1 Inside view is luxury, i love it</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>20 / MOQ 100 Nice worker answered all questions</t>
         </is>
@@ -2611,20 +2846,25 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
           <t>80 rmb for 230 meter</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>1560 rmb for whole item</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>4600 rmb</t>
         </is>
@@ -2641,20 +2881,25 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
@@ -2675,20 +2920,25 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
           <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>150 Yuan, 1 bottle. ( Taste is strong and good</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Haven't discussed the prices. Just got the company name list for future referenc</t>
         </is>
@@ -2725,20 +2975,25 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
           <t>2085</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>2147</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>2223</t>
         </is>
@@ -2775,20 +3030,25 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>General</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
           <t>250¥/м3</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>4500¥</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>8790$</t>
         </is>
@@ -2825,20 +3085,25 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
           <t>300¥ 300pcs</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>50¥ 1000pcs</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>500$ 100psc</t>
         </is>
@@ -2875,20 +3140,25 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
           <t>4500¥</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>8790$</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>250¥/m3</t>
         </is>
@@ -2921,20 +3191,25 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
           <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>1p, 10000$m2, very beautiful big red door</t>
         </is>
@@ -2971,20 +3246,25 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
           <t>1 container (400 square meters), 60 dollars for 1 square meters</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>Moq is 1 door, 530 RMB for 1 door</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>14400 dollars, moq - 1</t>
         </is>
@@ -3017,20 +3297,25 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
+          <t>Doors</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
           <t>1 товаров</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
         </is>
@@ -3063,20 +3348,25 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
           <t>100 RMB per sample. The taste is very good</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>150 RMB per sample. The taste is very good</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>250 RMB per sample. The taste is very good</t>
         </is>
@@ -3097,20 +3387,25 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
           <t>498rmb/unit. I like the green tea in white color. First time to see colorless te</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>The 中国好水 brand water was really good. They are using deep water instead of shall</t>
         </is>
@@ -3147,20 +3442,25 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
           <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="J60" t="inlineStr">
         <is>
           <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
         </is>
@@ -3197,20 +3497,25 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="J61" t="inlineStr">
         <is>
           <t>1050</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>550</t>
         </is>
@@ -3227,20 +3532,25 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
           <t>Prices are go and packing and Verstaliy is more</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>The taste anaroma is good of this product then anyother</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>the product prices are very good. looks attractive</t>
         </is>
@@ -3273,20 +3583,25 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
           <t>820 rmb moq 100</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>650 moq 300</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>560 moq 200</t>
         </is>
@@ -3323,20 +3638,25 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
           <t>2.5 RMB per unit, MOQ is 500 pieces. The plastic material was high quality and c</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this com</t>
         </is>
@@ -3369,20 +3689,25 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
           <t>1299, MOQ 200. I like the company and people there . Very friendly and know thei</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>5000rmb MOQ 50</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>1500 rmb MOQ 100</t>
         </is>
@@ -3415,20 +3740,25 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
           <t>Black matt tap water $20</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="J66" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t>109</t>
         </is>
@@ -3465,20 +3795,25 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
           <t>9$</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="J67" t="inlineStr">
         <is>
           <t>13.25$</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t>8.83$</t>
         </is>
@@ -3507,20 +3842,25 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
           <t>640 PCs, 3.72 RMB very good</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="J68" t="inlineStr">
         <is>
           <t>30 PCs, 420 RMB, need check quality</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="K68" t="inlineStr">
         <is>
           <t>10 PCs, 1150 RMB, very good</t>
         </is>
@@ -3553,20 +3893,25 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
           <t>10000</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="J69" t="inlineStr">
         <is>
           <t>10000</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="K69" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -3603,20 +3948,25 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
           <t>Depend on item</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="J70" t="inlineStr">
         <is>
           <t>Depend of quantity</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="K70" t="inlineStr">
         <is>
           <t>100/square meter</t>
         </is>
@@ -3653,20 +4003,25 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
           <t>RMB 15705 MOQ5; pleasant impression</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>MOQ5 25799 RMB</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t>RMB 19479; MOQ 1</t>
         </is>
@@ -3703,20 +4058,25 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="J72" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="K72" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
@@ -3753,20 +4113,25 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
           <t>2000$, can be customized, very convenient</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>38$, very unique</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>2050 rmb, very interesting, convenient to use for pets</t>
         </is>
@@ -3795,20 +4160,25 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
           <t>25 rmb, 1 box, like this product</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>34 rmb, 1000, normal</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>40 rmb, 2000, very good</t>
         </is>
@@ -3845,20 +4215,25 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
           <t>1 container 250 rmb</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="J75" t="inlineStr">
         <is>
           <t>1 container 500 rmb</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="K75" t="inlineStr">
         <is>
           <t>1 container 700 rmb</t>
         </is>
@@ -3895,20 +4270,25 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
           <t>Жду коммерческое предложение. Компания понравилась</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="J76" t="inlineStr">
         <is>
           <t>Цена зависит от обьема, от 3 юаней, расходники</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="K76" t="inlineStr">
         <is>
           <t>Прайс отправят, от 100ед, хорошая компания</t>
         </is>

</xml_diff>

<commit_message>
CBD catalog: add emails, remove duplicates, clean empty rows
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,40 +434,45 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Categories</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Comment 1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Comment 2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Comment 3</t>
         </is>
@@ -489,40 +494,45 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>crystal@sunhohiglobal.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>+86-137 0262 5097</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>www.sunhohiwindow.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>20th Floor, Building A1, Full International Financial Center, No. 28, Haiwu Road, Guicheng Street, Nanhai District, Foshan City, Guangdong Province, China</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>50.000¥. Moq-1</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>50.000¥. Moq-1</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>50.000¥. Moq-1</t>
         </is>
@@ -537,27 +547,28 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>500 pcs price 58 usd</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>1000 pcs price 120 usd</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>1000 pcs price 38 USD</t>
         </is>
@@ -579,40 +590,45 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>export01@gznewhoo.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>+86-198-7837-3626</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>www.gznewhoo.com</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Building 7, Hongyu Smart Industrial Park, No. 333 Juhuashi Avenue, Huadu District, Guangzhou</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>80$</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>70$</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>300 yuan</t>
         </is>
@@ -634,40 +650,45 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>kim.lok@bweetech.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>186-5759-0678</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>www.bweetech.com</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>上海市松江区沪亭北路99弄金地广场1号楼7层 (F7, #1, Plaza Jindi, Lane 99, North Huting Rd, Songjiang District, Shanghai)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Smart</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>500pcs / $100USD for pcs</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>50pcs / $50USD for pcs</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>20pcs / $100USD for pcs</t>
         </is>
@@ -689,36 +710,41 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>sales5@deiouxwindows.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>+86-13392246940</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>WWW.DEIOUXWINDOWS.COM</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>Custom order</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Custom order</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Custom order</t>
         </is>
@@ -740,40 +766,45 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>market@smarteklock.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>+86-15889896019</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>www.smarteklock.com</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>6F, Bldg 10, No.1 Shengyu Rd.Jidonger, Xiaolan Town, Zhongshan City, Guangdong, China 528415</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>170 to 335 usd</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>100 to up</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>100 to up usd</t>
         </is>
@@ -788,27 +819,28 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Coatings</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>Super</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Super</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Super</t>
         </is>
@@ -830,36 +862,41 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>sales03@cn-xindong.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>0086-182 5765 3405</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>Xuanmen Industrial Zone, Yuhuan, Zhejiang, China, 317608</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>50</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -881,36 +918,41 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>sales09@ouhuadec.comkindell1771@gmail.com962460055@qq.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>13326792105</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>佛山市南海区大沥谭边工业区虹岭一路一号（2号厂房）</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>Wall sheet , 200 rmb per meter , 2000 mtr,</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Handles , 500 moq , 100 rmb per handle</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Wall sheet and wooden wall sheet , 2000mtr , 150 rmb per mtr</t>
         </is>
@@ -932,40 +974,45 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>jinjian19@jinjianlock.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>15057304393</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>www.jinjianlock.com</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>温州市瓯海区郭溪街道智能锁具产业园(1号楼)1号</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>Price: 800 – 2600 CNY per unit depending on the model and features. MOQ: 100 uni</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Price: 1200 – 3500 CNY per unit depending on materials and security specificatio</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Price: 1800 – 4500 CNY per unit based on the finish and decorative complexity. M</t>
         </is>
@@ -985,38 +1032,39 @@
           <t>赖华芳</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>13727479513, 400-8339513</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>广东省佛山市顺德区龙江镇联塑嘉园三路3号9513家具总部</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Furnishing</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>3 товаров</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>Хорошее, 400rmb</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Хорошее , 1500rmb</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Нормальное</t>
         </is>
@@ -1028,36 +1076,57 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>中山市福乐门智能科技有限公司</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>CHINA GUANGCHAO CONTAINER HOUSE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>陈洁玲 Rowling</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>014@cgchcontainer.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>+86 189 2997 1329</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>www.cgchcontainer.com</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Rm. 5710, 656 Huangpu Ave., Tianhe, Guangzhou</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>$176, MOQ 50, very good!</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>$55, MOQ100pcs, good</t>
+          <t>1000 yuan 1 square</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>$30, MOQ 10pcs, nice</t>
+          <t>150 rmb</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>570 rmb</t>
         </is>
       </c>
     </row>
@@ -1067,52 +1136,57 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CHINA GUANGCHAO CONTAINER HOUSE</t>
+          <t>广东招材建材科技有限公司</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>陈洁玲 Rowling</t>
+          <t>黎桃桃</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+86 189 2997 1329</t>
+          <t>toto.liblun@gmail.com</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>www.cgchcontainer.com</t>
+          <t>+8618934320539</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Rm. 5710, 656 Huangpu Ave., Tianhe, Guangzhou</t>
+          <t>www.liblun.com</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>广东省佛山市南海区罗村社区新下村5号厂房</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1000 yuan 1 square</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>150 rmb</t>
+          <t>620 super</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>570 rmb</t>
+          <t>1500 super</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>130 super</t>
         </is>
       </c>
     </row>
@@ -1122,52 +1196,57 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>广东招材建材科技有限公司</t>
+          <t>广东伟经家居制品有限公司 (Guangdong Wireking Household Products Co., Ltd.)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>黎桃桃</t>
+          <t>欧阳玉滢 (Sonia Ouyang)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+8618934320539</t>
+          <t>sonia.ouyang@wireking.com</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>www.liblun.com</t>
+          <t>+86-13392758223</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区罗村社区新下村5号厂房</t>
+          <t>www.wireking.com</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Decoration</t>
+          <t>广东省佛山市顺德区均安镇智安北路12号 (No.12 Zhi'an North Road, Jun'an, Shunde, Foshan, Guangdong, China)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>620 super</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1500 super</t>
+          <t>$32, MOQ 300, good</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>130 super</t>
+          <t>¥3000, MoQ 1pcs, very good</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>¥17, Moq 50, good</t>
         </is>
       </c>
     </row>
@@ -1177,52 +1256,57 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>广东伟经家居制品有限公司 (Guangdong Wireking Household Products Co., Ltd.)</t>
+          <t>佛山市悠派家居科技有限公司</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>欧阳玉滢 (Sonia Ouyang)</t>
+          <t>黄伟业</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+86-13392758223</t>
+          <t>Yea@LGPKB.com</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>www.wireking.com</t>
+          <t>13825596371</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区均安镇智安北路12号 (No.12 Zhi'an North Road, Jun'an, Shunde, Foshan, Guangdong, China)</t>
+          <t>www.LGPKB.com</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>广东省佛山市顺德区大良街道古鉴成展路3号</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$32, MOQ 300, good</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>¥3000, MoQ 1pcs, very good</t>
+          <t>600 RMB Great, very cheap</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>¥17, Moq 50, good</t>
+          <t>800 rmb, little high</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>3400, Good price</t>
         </is>
       </c>
     </row>
@@ -1232,52 +1316,49 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>佛山市悠派家居科技有限公司</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>黄伟业</t>
-        </is>
-      </c>
+          <t>常州市永春保温材料有限公司</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>13825596371</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>www.LGPKB.com</t>
-        </is>
-      </c>
+          <t>yongchun1208@163.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道古鉴成展路3号</t>
+          <t>www.ycbwcl.1688.com</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>江苏省常州市</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>600 RMB Great, very cheap</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>800 rmb, little high</t>
+          <t>10$</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3400, Good price</t>
+          <t>69$</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>50-85$</t>
         </is>
       </c>
     </row>
@@ -1287,44 +1368,49 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>常州市永春保温材料有限公司</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>杭州班昇</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>陈卓敏 Ruby</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>295608376@qq.com</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>www.ycbwcl.1688.com</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>江苏省常州市</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Coatings</t>
-        </is>
-      </c>
+          <t>+86 13556688832</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>10$</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>69$</t>
+          <t>￥1000 good</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>50-85$</t>
+          <t>¥ 500 good</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>￥ 300 good</t>
         </is>
       </c>
     </row>
@@ -1334,44 +1420,45 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>杭州班昇</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>陈卓敏 Ruby</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>+86 13556688832</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>江门市新阳刚智能科技有限公司</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>135 3666 7789, 400-9090-518</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Decoration</t>
+          <t>广东省江门市新会区大泽镇万洋众创城38-1号</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>￥1000 good</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>¥ 500 good</t>
+          <t>300 rmb and more. Good quality and good price. Small quantity</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>￥ 300 good</t>
+          <t>33$ for 1 pcs. Good quality and quantity</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
         </is>
       </c>
     </row>
@@ -1381,44 +1468,45 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>江门市新阳刚智能科技有限公司</t>
+          <t>三强地毯 (THREE-STRONG CARPET)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>135 3666 7789, 400-9090-518</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>广东省江门市新会区大泽镇万洋众创城38-1号</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
+          <t>hengsheng_carpet@163.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0769-89807692</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>300 rmb and more. Good quality and good price. Small quantity</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>33$ for 1 pcs. Good quality and quantity</t>
+          <t>Good 👍</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
+          <t>1570</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>5800</t>
         </is>
       </c>
     </row>
@@ -1428,40 +1516,57 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>三强地毯 (THREE-STRONG CARPET)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>Zhejiang Kehon Intelligent Science &amp; Technology Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sammi Shi</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0769-89807692</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+          <t>sales01@kehon.cn</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>+86 156 8948 5097</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>www.kehon.cn</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Bath</t>
+          <t>No.1 Hangchuan Rd., Huzhen Town, Jinyun County, Zhejiang, China</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Good 👍</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1570</t>
+          <t>130 yuan</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>20000usd</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>500yuan</t>
         </is>
       </c>
     </row>
@@ -1471,52 +1576,57 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Zhejiang Kehon Intelligent Science &amp; Technology Co., Ltd.</t>
+          <t>CAE SANITARY FITTINGS INDUSTRY CO., LTD. GUANGDONG</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sammi Shi</t>
+          <t>Josie Guan</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>+86 156 8948 5097</t>
+          <t>cae@china-cae.com</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>www.kehon.cn</t>
+          <t>+86-13702279135</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>No.1 Hangchuan Rd., Huzhen Town, Jinyun County, Zhejiang, China</t>
+          <t>www.china-cae.com</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>No.62-64, Xingda Rd., Shagang Dist., ShuikouTown, Kaiping; Guangdong, P.R.Of China. PC: 529321</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>130 yuan</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>20000usd</t>
+          <t>MOQ 100, 47 rnb per piece</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>500yuan</t>
+          <t>MOQ 50, 200 rnb per</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>MOQ 10, 845 per piece</t>
         </is>
       </c>
     </row>
@@ -1526,52 +1636,57 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAE SANITARY FITTINGS INDUSTRY CO., LTD. GUANGDONG</t>
+          <t>利亚德光电股份有限公司</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Josie Guan</t>
+          <t>金厚强</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>+86-13702279135</t>
+          <t>jinhouqiang@leyard.com</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>www.china-cae.com</t>
+          <t>13510009569, 18829341125, 400-8592-666</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>No.62-64, Xingda Rd., Shagang Dist., ShuikouTown, Kaiping; Guangdong, P.R.Of China. PC: 529321</t>
+          <t>www.leyard.com</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>北京市海淀区颐和园路北正红旗西街9号 / 深圳市龙华区观澜街道君子布社区观和路6号利亚德南方产业园A栋</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>MOQ 100, 47 rnb per piece</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>MOQ 50, 200 rnb per</t>
+          <t>1pcs. Start from 60rmb. Novative technology</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>MOQ 10, 845 per piece</t>
+          <t>From 1pc. Natural materials.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>1250rmb. MOQ 1 pc</t>
         </is>
       </c>
     </row>
@@ -1581,52 +1696,57 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>利亚德光电股份有限公司</t>
+          <t>广州传祺时代智能科技有限公司</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>金厚强</t>
+          <t>洪美兰</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>13510009569, 18829341125, 400-8592-666</t>
+          <t>jiang@chuangqitimes.com</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>www.leyard.com</t>
+          <t>13450298606</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>北京市海淀区颐和园路北正红旗西街9号 / 深圳市龙华区观澜街道君子布社区观和路6号利亚德南方产业园A栋</t>
+          <t>www.chuangqitimes.com</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>广州市黄埔区云埔工业区观达路20号密博科技园</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1pcs. Start from 60rmb. Novative technology</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>From 1pc. Natural materials.</t>
+          <t>329</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1250rmb. MOQ 1 pc</t>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>680</t>
         </is>
       </c>
     </row>
@@ -1636,52 +1756,57 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Zhejiang Kehon Intelligent Science &amp; Technology Co.,Ltd.</t>
+          <t>Guangdong CAE Sanitary Fittings Co., Ltd.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Janice Kuan</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>+86 157 5573 4990</t>
+          <t>jack@cae.com.cn</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>www.kehon.cn</t>
+          <t>+86-750-2713118</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>No.1 Hangchuan Rd., Huzhen Town, Jinyun County, Zhejiang, China</t>
+          <t>www.cae.cn</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>No.22, 2nd Phase, Shuikou Sanitary Ware Industrial Park, Kaiping, Guangdong, China</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>150 yuan, 100, good range of products</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>800usd, very nice, good quality product</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Set of furniture is very good quality, I like the company has also a showroom in</t>
         </is>
       </c>
     </row>
@@ -1691,52 +1816,53 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>广州传祺时代智能科技有限公司</t>
+          <t>JNOD 基诺德</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>洪美兰</t>
+          <t>周信朋 Joe Zhou</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>13450298606</t>
+          <t>sales02@jnodwater.com</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>www.chuangqitimes.com</t>
+          <t>+86 199 2825 2201</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>广州市黄埔区云埔工业区观达路20号密博科技园</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+          <t>www.jnodwater.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>199</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -1746,52 +1872,53 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Guangdong CAE Sanitary Fittings Co., Ltd.</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Janice Kuan</t>
-        </is>
-      </c>
+          <t>榜威电子科技（上海）有限公司</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>+86-750-2713118</t>
+          <t>service@bweetech.com</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>www.cae.cn</t>
+          <t>021-57715805</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>No.22, 2nd Phase, Shuikou Sanitary Ware Industrial Park, Kaiping, Guangdong, China</t>
+          <t>www.bweetech.com</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>上海市闵行区新骏环路188号15号楼南5层A501室</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>150 yuan, 100, good range of products</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>800usd, very nice, good quality product</t>
+          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не р</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Set of furniture is very good quality, I like the company has also a showroom in</t>
+          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с е</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно за</t>
         </is>
       </c>
     </row>
@@ -1801,36 +1928,57 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>THOR索而</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+          <t>Suzhou Acousound New Material Technology Inc.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Yolanda He</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>acousound02@polyacoustic.com</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>+86-18018121056</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>www.polyacoustic.com</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>No.10 Aimin Road, Xiangcheng, Suzhou, Jiangsu, China 215152</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functio</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functio</t>
+          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного </t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>I couldn't tell you the price for smart pens right away, but they said they woul</t>
+          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количест</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккур</t>
         </is>
       </c>
     </row>
@@ -1840,48 +1988,57 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JNOD 基诺德</t>
+          <t>诺奥(福建)环保家居用品有限公司</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>周信朋 Joe Zhou</t>
+          <t>蔡绿缘</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>+86 199 2825 2201</t>
+          <t>wendyyian@163.com</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>www.jnodwater.com</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>0086-13599917696</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>www.fjnuoao.cn</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>福建省漳州市长泰区兴泰工业园区台湾工业园锦都路191号</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>2900 usd</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1891,48 +2048,57 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>榜威电子科技（上海）有限公司</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>Guangzhou Sunrans Sanitary Ware Co., Ltd / Guangzhou Sunrans New Energy Technology Co., Ltd</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>William</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>021-57715805</t>
+          <t>william@sunrans.com</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>www.bweetech.com</t>
+          <t>+86 134 1613 9887</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>上海市闵行区新骏环路188号15号楼南5层A501室</t>
+          <t>http://www.sunrans.com</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Headquarter: No.38-4, Lisan Avenue, Zengjiang Street, Zengcheng, Guangzhou; Factory: Xiang 2 Road, Huizhou Industrial Transfer Park, Huizhou, China 516820</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не р</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с е</t>
+          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product a</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно за</t>
+          <t>MOQ 1, they got samples. 8000usd. Very well made product, trendy and popular. Th</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable</t>
         </is>
       </c>
     </row>
@@ -1942,52 +2108,57 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Suzhou Acousound New Material Technology Inc.</t>
+          <t>IFUN PARK &amp; TIPTOPFUN AMUSEMENT</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Yolanda He</t>
+          <t>Ivy Zhou</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>+86-18018121056</t>
+          <t>ivy@ifunpark.com</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>www.polyacoustic.com</t>
+          <t>+86 133 0238 5758</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>No.10 Aimin Road, Xiangcheng, Suzhou, Jiangsu, China 215152</t>
+          <t>www.ifunpark.com / www.ifunamusement.com</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>No. 13, Wenqiao Road, Xinqiao Village, Shiji Town, Panyu District, Guangzhou City, China</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Decoration</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного </t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количест</t>
+          <t>600</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккур</t>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -1997,52 +2168,57 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>诺奥(福建)环保家居用品有限公司</t>
+          <t>RENQIU TUOXIN BUILDING MATERIALS CO., LTD</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>蔡绿缘</t>
+          <t>Emily Li</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0086-13599917696</t>
+          <t>tuoxinlqm@outlook.com</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>www.fjnuoao.cn</t>
+          <t>+86 19831737599</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>福建省漳州市长泰区兴泰工业园区台湾工业园锦都路191号</t>
+          <t>https://www.tuoxinfiberglassmesh.com/</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Bath</t>
+          <t>Yanling Industrial Park, Renqiu City, Hebei Province, China</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2900 usd</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0.6 usd/m2</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Under negotiation, great opportunities</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>1-5 usd/l</t>
         </is>
       </c>
     </row>
@@ -2052,52 +2228,53 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Guangzhou Sunrans Sanitary Ware Co., Ltd / Guangzhou Sunrans New Energy Technology Co., Ltd</t>
+          <t>安居福智能门</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>罗加玲</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>+86 134 1613 9887</t>
+          <t>1040857731@qq.com</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>http://www.sunrans.com</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Headquarter: No.38-4, Lisan Avenue, Zengjiang Street, Zengcheng, Guangzhou; Factory: Xiang 2 Road, Huizhou Industrial Transfer Park, Huizhou, China 516820</t>
-        </is>
-      </c>
+          <t>18928121650</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bath</t>
+          <t>广东省中山市东凤镇</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product a</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>MOQ 1, they got samples. 8000usd. Very well made product, trendy and popular. Th</t>
+          <t>100</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable</t>
+          <t>679 rmb</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>59 rmb</t>
         </is>
       </c>
     </row>
@@ -2107,52 +2284,41 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IFUN PARK &amp; TIPTOPFUN AMUSEMENT</t>
+          <t>东方喜卡</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ivy Zhou</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>+86 133 0238 5758</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>www.ifunpark.com / www.ifunamusement.com</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>No. 13, Wenqiao Road, Xinqiao Village, Shiji Town, Panyu District, Guangzhou City, China</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Decoration</t>
-        </is>
-      </c>
+          <t>果果</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>249RMB</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>6000RMB</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2000RMB&amp;gt;</t>
         </is>
       </c>
     </row>
@@ -2162,52 +2328,53 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RENQIU TUOXIN BUILDING MATERIALS CO., LTD</t>
+          <t>GUANGDONG TUOXUN INTELLIGENT TECHNOLOGY CO., LTD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Emily Li</t>
+          <t>Wing</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>+86 19831737599</t>
+          <t>wuyunying08@gmail.com</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.tuoxinfiberglassmesh.com/</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Yanling Industrial Park, Renqiu City, Hebei Province, China</t>
-        </is>
-      </c>
+          <t>189-2984-9818</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
+          <t>Auto Parts Industrial Park, Jinli Town, Gaoyao District, Zhaoqing, Guangdong</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>0.6 usd/m2</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Under negotiation, great opportunities</t>
+          <t>MOQ - 5000 and price - 7000 dollars</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1-5 usd/l</t>
+          <t>4000$</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>3000 dollars</t>
         </is>
       </c>
     </row>
@@ -2217,48 +2384,53 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>安居福智能门</t>
+          <t>佛山市方泓五金建材有限公司</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>罗加玲</t>
+          <t>陈施志凯</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>18928121650</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>广东省中山市东凤镇</t>
-        </is>
-      </c>
+          <t>108455453@qq.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>+86 134 3318 1558</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
+          <t>中国广东省佛山市南海区里水镇大步工业区13号</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>679 rmb</t>
+          <t>The price cheap, merchant very friendly</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>59 rmb</t>
+          <t>The price more cheaper, good quality</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Good merchant, perfect products</t>
         </is>
       </c>
     </row>
@@ -2268,40 +2440,57 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>东方喜卡</t>
+          <t>Gaocheng</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>果果</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
+          <t>叶小龙/Dustin Ye</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>yedustin@gmail.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>+86-188 5861 0008</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>www.cngaocheng.cn</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>浙江省三门县浦坝港镇沿海工业城 (Coastal Industrial City, Pubagang Town, Sanmen, Taizhou City, Zhejiang Pro., China)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>249RMB</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>6000RMB</t>
+          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their produc</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2000RMB&amp;gt;</t>
+          <t>15 RMB the product is interesting</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>nearly $15,000 for this production line</t>
         </is>
       </c>
     </row>
@@ -2311,48 +2500,57 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GUANGDONG TUOXUN INTELLIGENT TECHNOLOGY CO., LTD</t>
+          <t>ZHEJIANG DOUBLE-LIN VALVES CO., LTD.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Wing</t>
+          <t>Dream Lin</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>189-2984-9818</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+          <t>sale15@double-lin.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>86-13710718529, 86-020-66837727</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Auto Parts Industrial Park, Jinli Town, Gaoyao District, Zhaoqing, Guangdong</t>
+          <t>www.double-lin.com</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
+          <t>Yanpan Hardware Industrial Area, Ganjiang Town, Yuhuan, Zhejiang, China</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>MOQ - 5000 and price - 7000 dollars</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>4000$</t>
+          <t>149</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>3000 dollars</t>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>749</t>
         </is>
       </c>
     </row>
@@ -2362,48 +2560,57 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>佛山市方泓五金建材有限公司</t>
+          <t>CHANGZHOU YOUCARE DECORATION ENGINEERING CO.LTD.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>陈施志凯</t>
+          <t>Eric Huang</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>+86 134 3318 1558</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+          <t>464565801@qq.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>13813551160, 0519-88784050</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>中国广东省佛山市南海区里水镇大步工业区13号</t>
+          <t>www.ycpanel.com</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>#28, Changzhou East Road, Henglin Town, Changzhou City, Jiangsu, China</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>The price cheap, merchant very friendly</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>The price more cheaper, good quality</t>
+          <t>5000 USD</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Good merchant, perfect products</t>
+          <t>3000 USD</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>3000 USD</t>
         </is>
       </c>
     </row>
@@ -2413,52 +2620,41 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Gaocheng</t>
+          <t>优品声学吸音隔音</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>叶小龙/Dustin Ye</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>+86-188 5861 0008</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>www.cngaocheng.cn</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>浙江省三门县浦坝港镇沿海工业城 (Coastal Industrial City, Pubagang Town, Sanmen, Taizhou City, Zhejiang Pro., China)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Bath</t>
-        </is>
-      </c>
+          <t>杨伟杰</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their produc</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>15 RMB the product is interesting</t>
+          <t>6000 RMB. I like the way they explain everything about their product.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>nearly $15,000 for this production line</t>
+          <t>Smart home system 2000 RMB. They have showed us how the smart home system works.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>249 RMB. They have fully described their products.</t>
         </is>
       </c>
     </row>
@@ -2468,52 +2664,45 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ZHEJIANG DOUBLE-LIN VALVES CO., LTD.</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Dream Lin</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>86-13710718529, 86-020-66837727</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>www.double-lin.com</t>
-        </is>
-      </c>
+          <t>广州市优品声学科技有限公司</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Yanpan Hardware Industrial Area, Ganjiang Town, Yuhuan, Zhejiang, China</t>
+          <t>www.gzypsx.com</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>广东省广州市番禺区石碁镇文边路28号二栋二层</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>6000RMB，积极，详细地告诉了一切</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>249RMB , 价格很便宜</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2000 RMB</t>
         </is>
       </c>
     </row>
@@ -2523,52 +2712,53 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CHANGZHOU YOUCARE DECORATION ENGINEERING CO.LTD.</t>
+          <t>贵州佑远木业有限公司</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eric Huang</t>
+          <t>颜加伟</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>13813551160, 0519-88784050</t>
+          <t>1164199388@qq.com</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>www.ycpanel.com</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>#28, Changzhou East Road, Henglin Town, Changzhou City, Jiangsu, China</t>
-        </is>
-      </c>
+          <t>133 9983 5678</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Decoration</t>
+          <t>贵州省赤水市成渝（赤水）家具产业园A3-2</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Coatings</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>5000 USD</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>3000 USD</t>
+          <t>400rmb /m2 good meeting</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>3000 USD</t>
+          <t>350 rmb/m2</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>MOQ 5000 pieces</t>
         </is>
       </c>
     </row>
@@ -2578,40 +2768,57 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>优品声学吸音隔音</t>
+          <t>MOERSHU 摩尔舒卫浴</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>杨伟杰</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
+          <t>Thea</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>moershu3@moershu.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>13957622087</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>www.moershu.com</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>777 Shanzhuan Road, Zhujiajiao Industrial Park, Qingpu District, Shanghai, China; No. 399 Haiyun Road, Jiaojiang District, Taizhou City, Zhejiang Province, China; 88-3 East Taihe Road, Jiaojiang District, Taizhou City, Zhejiang Province, China</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>6000 RMB. I like the way they explain everything about their product.</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Smart home system 2000 RMB. They have showed us how the smart home system works.</t>
+          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>249 RMB. They have fully described their products.</t>
+          <t>3000 / MOQ 1 Inside view is luxury, i love it</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>20 / MOQ 100 Nice worker answered all questions</t>
         </is>
       </c>
     </row>
@@ -2621,44 +2828,53 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>广州市优品声学科技有限公司</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+          <t>江西荣科新型材料有限公司 (JIANGXI RONGKE NEW BUILDING MATERIALS CO., LTD)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lucy Zeng (曾露)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>lucy@rongkedecor.com</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>www.gzypsx.com</t>
+          <t>+86-13134020034</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>广东省广州市番禺区石碁镇文边路28号二栋二层</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Doors</t>
-        </is>
-      </c>
+          <t>https://www.amerdecor.com/</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>6000RMB，积极，详细地告诉了一切</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>249RMB , 价格很便宜</t>
+          <t>80 rmb for 230 meter</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2000 RMB</t>
+          <t>1560 rmb for whole item</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>4600 rmb</t>
         </is>
       </c>
     </row>
@@ -2666,50 +2882,35 @@
       <c r="A45" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>贵州佑远木业有限公司</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>颜加伟</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>133 9983 5678</t>
-        </is>
-      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>贵州省赤水市成渝（赤水）家具产业园A3-2</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Coatings</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400rmb /m2 good meeting</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>350 rmb/m2</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>MOQ 5000 pieces</t>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -2719,48 +2920,53 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>贵州佑远木业有限公司</t>
+          <t>江西瑞京鸿兴实业有限公司</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>颜加伟</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>133 9983 5678</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr"/>
+          <t>朱友群</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>13763963598</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>贵州省赤水市成渝(赤水)家居产业园A3-2</t>
+          <t>www.jx-wpc.com</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Coatings</t>
+          <t>江西省瑞金市经济开发区创业一路东侧</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>General</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>400rmb/m2</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>350rmb/m2</t>
+          <t>250¥/м3</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>MOQ 5000 pieces</t>
+          <t>4500¥</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>8790$</t>
         </is>
       </c>
     </row>
@@ -2770,52 +2976,57 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MOERSHU 摩尔舒卫浴</t>
+          <t>ciarra</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Thea</t>
+          <t>Linda</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>13957622087</t>
+          <t>linda.lu@ciarrahome.com</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>www.moershu.com</t>
+          <t>+86 1882 9964 960 / +86 1343 2639 580</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>777 Shanzhuan Road, Zhujiajiao Industrial Park, Qingpu District, Shanghai, China; No. 399 Haiyun Road, Jiaojiang District, Taizhou City, Zhejiang Province, China; 88-3 East Taihe Road, Jiaojiang District, Taizhou City, Zhejiang Province, China</t>
+          <t>www.ciarrahome.com</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Bath</t>
+          <t>Poly Center, Room 1703, 5 Linjiang Avenue, Tianhe, Guangzhou, Guangdong, China, 510623</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>3000 / MOQ 1 Inside view is luxury, i love it</t>
+          <t>300¥ 300pcs</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>20 / MOQ 100 Nice worker answered all questions</t>
+          <t>50¥ 1000pcs</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>500$ 100psc</t>
         </is>
       </c>
     </row>
@@ -2825,48 +3036,57 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>江西荣科新型材料有限公司 (JIANGXI RONGKE NEW BUILDING MATERIALS CO., LTD)</t>
+          <t>Xuancheng Hengxin Sanitary Ware Co., Ltd</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Lucy Zeng (曾露)</t>
+          <t>Anne</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>+86-13134020034</t>
+          <t>victor@ck-bath.com</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.amerdecor.com/</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>18656330093</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://ck-bath.com/</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Yangyin Avenue, Xiangyang Town, Xuanzhou District, Xuancheng City, Anhui Province</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>80 rmb for 230 meter</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>1560 rmb for whole item</t>
+          <t>4500¥</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>4600 rmb</t>
+          <t>8790$</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>250¥/m3</t>
         </is>
       </c>
     </row>
@@ -2874,34 +3094,55 @@
       <c r="A49" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>佛山市旌晨铝门窗有限公司</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>胡光辉</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1525423805@qq.com</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>18128752879</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>佛山市狮山镇谭边工业区崩岗头路四号之一</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>1p, 10000$m2, very beautiful big red door</t>
         </is>
       </c>
     </row>
@@ -2911,36 +3152,57 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>东风汽车</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+          <t>河南贝迪塑业有限公司 (HENAN BEIDI PLASTIC INDUSTRY CO., LTD.)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>代桂菊 (Cathy Dai)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>cathy@hnbeidi.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>+86 151 3737 2072</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>www.baydeegroup.com</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>中国河南省鹤壁市 (HEBI CITY, HENAN PROVINCE, CHINA)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>150 Yuan, 1 bottle. ( Taste is strong and good</t>
+          <t>1 container (400 square meters), 60 dollars for 1 square meters</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Haven't discussed the prices. Just got the company name list for future referenc</t>
+          <t>Moq is 1 door, 530 RMB for 1 door</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>14400 dollars, moq - 1</t>
         </is>
       </c>
     </row>
@@ -2950,52 +3212,49 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CHANGZHOU YOUCARE DECORATION ENGINEERING CO.,LTD.</t>
+          <t>景德镇窑珍陶瓷</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Eric Huang</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>13813551160</t>
-        </is>
-      </c>
+          <t>徐云霞</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>www.ycpanel.com</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>#28. Changzhou East Road, Henglin Town, Changzhou City, Jiangsu, China</t>
-        </is>
-      </c>
+          <t>13697981203</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Decoration</t>
+          <t>店面地址：江西省景德镇市国贸广场国贸街1号；厂址：吕蒙高新工业园沟上008号</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Furnishing</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2085</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2147</t>
+          <t>100 RMB per sample. The taste is very good</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>150 RMB per sample. The taste is very good</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>250 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -3005,52 +3264,57 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>江西瑞京鸿兴实业有限公司</t>
+          <t>聖羅蘭·衛浴 (Sannora)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>朱友群</t>
+          <t>ALLEN XU (许熙平)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>13763963598</t>
+          <t>sales5@sannora.com</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>www.jx-wpc.com</t>
+          <t>+86 137 0224 0244</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>江西省瑞金市经济开发区创业一路东侧</t>
+          <t>www.sannora.com</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Tangxia Ind. Zone, Shishan Town, Nanhai Dist., Foshan, Guangdong, China</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>250¥/м3</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>4500¥</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>8790$</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
         </is>
       </c>
     </row>
@@ -3060,52 +3324,57 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ciarra</t>
+          <t>ZHEJIANG SEATING TECHNOLOGY CO., LTD.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>May Zhang</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>+86 1882 9964 960 / +86 1343 2639 580</t>
+          <t>sales5@anjeurostilefurniture.com</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>www.ciarrahome.com</t>
+          <t>+86 182 5727 1590</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Poly Center, Room 1703, 5 Linjiang Avenue, Tianhe, Guangzhou, Guangdong, China, 510623</t>
+          <t>www.zjseating.com</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
+          <t>150 Taining Road, TianZiHu Industrial Area, Anji, Huzhou, Zhejiang, China. Post Code: 313300</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
           <t>Furnishing</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>300¥ 300pcs</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>50¥ 1000pcs</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>500$ 100psc</t>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>550</t>
         </is>
       </c>
     </row>
@@ -3113,54 +3382,35 @@
       <c r="A54" t="n">
         <v>53</v>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Xuancheng Hengxin Sanitary Ware Co., Ltd</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Anne</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>18656330093</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>https://ck-bath.com/</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Yangyin Avenue, Xiangyang Town, Xuanzhou District, Xuancheng City, Anhui Province</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Bath</t>
-        </is>
-      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>4500¥</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>8790$</t>
+          <t>Prices are go and packing and Verstaliy is more</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>250¥/m3</t>
+          <t>The taste anaroma is good of this product then anyother</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>the product prices are very good. looks attractive</t>
         </is>
       </c>
     </row>
@@ -3170,48 +3420,57 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>佛山市旌晨铝门窗有限公司</t>
+          <t>HONGKONG PINGAO INDUSTRIAL CO., LTD / PINGAO HARDWARE &amp; PLASTIC PRODUCTS FACTORY</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>胡光辉</t>
+          <t>Pacao Yin</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>18128752879</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
+          <t>pin@pingaolao.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>(0086)13903035682 / (0086)0769-86378283</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>佛山市狮山镇谭边工业区崩岗头路四号之一</t>
+          <t>www.pingaolao.com / https://dgpingao.1688.com</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>NO.5 JINTAN SECOND STREET, SHANGWU INDUSTRIAL, SHIJIE TOWN, DONGGUAN, GUANGDONG, CHINA</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
+          <t>2.5 RMB per unit, MOQ is 500 pieces. The plastic material was high quality and c</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>1p, 10000$m2, very beautiful big red door</t>
+          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this com</t>
         </is>
       </c>
     </row>
@@ -3221,52 +3480,57 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>河南贝迪塑业有限公司 (HENAN BEIDI PLASTIC INDUSTRY CO., LTD.)</t>
+          <t>Chongnuo(Shandong)NewMaterial Co.,Ltd.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>代桂菊 (Cathy Dai)</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>+86 151 3737 2072</t>
+          <t>sales06@chongnuo-floors.com</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>www.baydeegroup.com</t>
+          <t>+86 19906379675</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>中国河南省鹤壁市 (HEBI CITY, HENAN PROVINCE, CHINA)</t>
+          <t>www.chongnuo-floors.com</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>Qingyun County, Dezhou City, China</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>1 container (400 square meters), 60 dollars for 1 square meters</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Moq is 1 door, 530 RMB for 1 door</t>
+          <t>9$</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>14400 dollars, moq - 1</t>
+          <t>13.25$</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>8.83$</t>
         </is>
       </c>
     </row>
@@ -3276,48 +3540,45 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>佛山市旌晨铝门窗有限公司</t>
+          <t>ZHE JIANG TIANYAN HOLDING LTD</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>张广帅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>13726358587, 400-9155262</t>
-        </is>
-      </c>
+          <t>NICOLE</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>佛山市狮山镇谭边工业区顾岗头路四号之一</t>
-        </is>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>TAIZHOU, ZHEJIANG</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
+          <t>640 PCs, 3.72 RMB very good</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается </t>
+          <t>30 PCs, 420 RMB, need check quality</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>10 PCs, 1150 RMB, very good</t>
         </is>
       </c>
     </row>
@@ -3327,48 +3588,53 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>景德镇窑珍陶瓷</t>
+          <t>中国广东柜邦精密金属制品有限公司 (China Guangdong Guibang Precision Metal Products Co.Ltd)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>徐云霞</t>
+          <t>唐一智 (JUNIOR)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>13697981203</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>店面地址：江西省景德镇市国贸广场国贸街1号；厂址：吕蒙高新工业园沟上008号</t>
-        </is>
-      </c>
+          <t>13621417@QQ.COM</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>+86-156-2562-1155</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Furnishing</t>
+          <t>Jieyang City, Guangdong Province Jiedong Longwei high-tech Zone industrial Park</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>100 RMB per sample. The taste is very good</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>150 RMB per sample. The taste is very good</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>250 RMB per sample. The taste is very good</t>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -3378,36 +3644,57 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>湖北龙王垭茶业有限公司</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
+          <t>广东亚当斯金属精密制造有限公司 (Guangdong Adams Metal Precision Manufacturing Co., Ltd.)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Kelly Liang 梁凯莹</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>kelly@adamsmetal.com.cn</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>+86-180-2935-2895 / +86-757-25331912</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>www.adamsmetal.com.cn</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>广东省佛山市顺德区勒流镇港口路10号 (No.10, Gangkou Road, Leliu Town, Shunde District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>498rmb/unit. I like the green tea in white color. First time to see colorless te</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks</t>
+          <t>Depend on item</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>The 中国好水 brand water was really good. They are using deep water instead of shall</t>
+          <t>Depend of quantity</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>100/square meter</t>
         </is>
       </c>
     </row>
@@ -3417,52 +3704,57 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>聖羅蘭·衛浴 (Sannora)</t>
+          <t>多彩帐篷 (DUOCAI TENT)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ALLEN XU (许熙平)</t>
+          <t>Jimmy 黄锦民</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>+86 137 0224 0244</t>
+          <t>sales003@sdduocaizp.com</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>www.sannora.com</t>
+          <t>+86-766-8298662, (86)133 2294 8506</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Tangxia Ind. Zone, Shishan Town, Nanhai Dist., Foshan, Guangdong, China</t>
+          <t>www.dc-tent.com, www.sdduocaizp.com</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Bath</t>
+          <t>广东省云浮市云安区佛山(云浮)产业转移工业园86号 / No.86 Foshan(Yunfu) Industrial transfer park, Yunan, Yunfu, Guangdong, China</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
+          <t>RMB 15705 MOQ5; pleasant impression</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inqui</t>
+          <t>MOQ5 25799 RMB</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>RMB 19479; MOQ 1</t>
         </is>
       </c>
     </row>
@@ -3472,52 +3764,57 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ZHEJIANG SEATING TECHNOLOGY CO., LTD.</t>
+          <t>河北天丰金属制品有限公司 (Hebei Tianfeng Metal Products Co., Ltd.)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>May Zhang</t>
+          <t>孟少美 (Elie Meng)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>+86 182 5727 1590</t>
+          <t>boilide.hinge@163.comxujianzhai1987@qq.com13621417@qq.comtff@hbtfjs.comkelly@adamsmetal.com.cnjane@dirock.cn</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>www.zjseating.com</t>
+          <t>13103196326</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>150 Taining Road, TianZiHu Industrial Area, Anji, Huzhou, Zhejiang, China. Post Code: 313300</t>
+          <t>www.hbtfjs.com</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Furnishing</t>
+          <t>河北省隆尧县公子村工业区 (Gongzi Village Industry Zone, Longyao County, Xingtai City, Hebei, China)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -3525,34 +3822,59 @@
       <c r="A62" t="n">
         <v>61</v>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>广州蒙娜丽莎卫浴股份有限公司</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>伍乐彤</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>monalisa702@monalisa.cn</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>86 13711117863</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>www.monalisa.cn</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>广州市花都区花东镇港头工业区4号</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Bath</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Prices are go and packing and Verstaliy is more</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>The taste anaroma is good of this product then anyother</t>
+          <t>2000$, can be customized, very convenient</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>the product prices are very good. looks attractive</t>
+          <t>38$, very unique</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2050 rmb, very interesting, convenient to use for pets</t>
         </is>
       </c>
     </row>
@@ -3562,48 +3884,45 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>佛山市同路匠人家具有限公司</t>
+          <t>广西中晨木业有限公司 (Guangxi Zhongchen Wood Industry Co., Ltd.)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>蒙玉婷</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>13160953218</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>广东省佛山市顺德区龙江镇联盟路三路3号9513家具总部</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Furnishing</t>
-        </is>
-      </c>
+          <t>张爱彬 (Zhang Aibin)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>+86 18178085851</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>820 rmb moq 100</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>650 moq 300</t>
+          <t>25 rmb, 1 box, like this product</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>560 moq 200</t>
+          <t>34 rmb, 1000, normal</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>40 rmb, 2000, very good</t>
         </is>
       </c>
     </row>
@@ -3613,52 +3932,57 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>HONGKONG PINGAO INDUSTRIAL CO., LTD / PINGAO HARDWARE &amp; PLASTIC PRODUCTS FACTORY</t>
+          <t>浙江安吉双虎竹木业有限公司</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pacao Yin</t>
+          <t>周瑶琳</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>(0086)13903035682 / (0086)0769-86378283</t>
+          <t>lisa.nordi@nuodibm.com</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>www.pingaolao.com / https://dgpingao.1688.com</t>
+          <t>+86-137 3822 8209</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>NO.5 JINTAN SECOND STREET, SHANGWU INDUSTRIAL, SHIJIE TOWN, DONGGUAN, GUANGDONG, CHINA</t>
+          <t>www.tigerbamboo.com / www.nuodibm.com</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>浙江省湖州市安吉县孝丰镇大竹村</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2.5 RMB per unit, MOQ is 500 pieces. The plastic material was high quality and c</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping</t>
+          <t>1 container 250 rmb</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this com</t>
+          <t>1 container 500 rmb</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>1 container 700 rmb</t>
         </is>
       </c>
     </row>
@@ -3668,627 +3992,55 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>佛山市同路匠人家具有限公司</t>
+          <t>宏宇集团 (HONGYU GROUP)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>肖汝兰</t>
+          <t>Melina 王玲</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>18675197017</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
+          <t>lina@hongyugroup.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>+86 13827702216</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区龙江镇联盟嘉园三路3号9513家具总部</t>
+          <t>en.hongyugroup.com</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Furnishing</t>
+          <t>广东省佛山市禅城区江湾二路26号 (No.26 Jiangwan Second Road, Chancheng District, Foshan, Guangdong)</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>3 товаров</t>
+          <t>Decoration</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>1299, MOQ 200. I like the company and people there . Very friendly and know thei</t>
+          <t>3 товаров</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>5000rmb MOQ 50</t>
+          <t>Жду коммерческое предложение. Компания понравилась</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>1500 rmb MOQ 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>浙江鑫东洁具有限公司 (ZHEJIANG XINDONG SANITARY WARE CO., LTD.)</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>冯晶晶 Joanna</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>0086-159 9067 6107</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Xuanmen Industrial Zone, Yuhuan, Zhejiang, China, 317608</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Black matt tap water $20</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>109</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Chongnuo(Shandong)NewMaterial Co.,Ltd.</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Daisy</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>+86 19906379675</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>www.chongnuo-floors.com</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Qingyun County, Dezhou City, China</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Decoration</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>9$</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>13.25$</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>8.83$</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>ZHE JIANG TIANYAN HOLDING LTD</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>NICOLE</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>TAIZHOU, ZHEJIANG</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>640 PCs, 3.72 RMB very good</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>30 PCs, 420 RMB, need check quality</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>10 PCs, 1150 RMB, very good</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>中国广东柜邦精密金属制品有限公司 (China Guangdong Guibang Precision Metal Products Co.Ltd)</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>唐一智 (JUNIOR)</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>+86-156-2562-1155</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Jieyang City, Guangdong Province Jiedong Longwei high-tech Zone industrial Park</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>广东亚当斯金属精密制造有限公司 (Guangdong Adams Metal Precision Manufacturing Co., Ltd.)</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Kelly Liang 梁凯莹</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>+86-180-2935-2895 / +86-757-25331912</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>www.adamsmetal.com.cn</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>广东省佛山市顺德区勒流镇港口路10号 (No.10, Gangkou Road, Leliu Town, Shunde District, Foshan City, Guangdong Province)</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Depend on item</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>Depend of quantity</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>100/square meter</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>多彩帐篷 (DUOCAI TENT)</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Jimmy 黄锦民</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>+86-766-8298662, (86)133 2294 8506</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>www.dc-tent.com, www.sdduocaizp.com</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>广东省云浮市云安区佛山(云浮)产业转移工业园86号 / No.86 Foshan(Yunfu) Industrial transfer park, Yunan, Yunfu, Guangdong, China</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Building</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>RMB 15705 MOQ5; pleasant impression</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>MOQ5 25799 RMB</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>RMB 19479; MOQ 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>河北天丰金属制品有限公司 (Hebei Tianfeng Metal Products Co., Ltd.)</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>孟少美 (Elie Meng)</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>13103196326</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>www.hbtfjs.com</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>河北省隆尧县公子村工业区 (Gongzi Village Industry Zone, Longyao County, Xingtai City, Hebei, China)</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>广州蒙娜丽莎卫浴股份有限公司</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>伍乐彤</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>86 13711117863</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>www.monalisa.cn</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>广州市花都区花东镇港头工业区4号</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Bath</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>2000$, can be customized, very convenient</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>38$, very unique</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>2050 rmb, very interesting, convenient to use for pets</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>广西中晨木业有限公司 (Guangxi Zhongchen Wood Industry Co., Ltd.)</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>张爱彬 (Zhang Aibin)</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>+86 18178085851</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Decoration</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>25 rmb, 1 box, like this product</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>34 rmb, 1000, normal</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>40 rmb, 2000, very good</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>浙江安吉双虎竹木业有限公司</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>周瑶琳</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>+86-137 3822 8209</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>www.tigerbamboo.com / www.nuodibm.com</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>浙江省湖州市安吉县孝丰镇大竹村</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>Decoration</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>1 container 250 rmb</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>1 container 500 rmb</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>1 container 700 rmb</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>宏宇集团 (HONGYU GROUP)</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Melina 王玲</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>+86 13827702216</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>en.hongyugroup.com</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>广东省佛山市禅城区江湾二路26号 (No.26 Jiangwan Second Road, Chancheng District, Foshan, Guangdong)</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Decoration</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>3 товаров</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>Жду коммерческое предложение. Компания понравилась</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
           <t>Цена зависит от обьема, от 3 юаней, расходники</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>Прайс отправят, от 100ед, хорошая компания</t>
         </is>

</xml_diff>

<commit_message>
CBD: fix 1 card + 1 product per supplier
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I182"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Super | 620 super</t>
+          <t>Super</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>130 super</t>
+          <t>620 super</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>$32, MOQ 300, good</t>
+          <t>1500 super</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>¥3000, MoQ 1pcs, very good</t>
+          <t>130 super</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>¥17, Moq 50, good</t>
+          <t>$32, MOQ 300, good</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>600 RMB Great, very cheap</t>
+          <t>¥3000, MoQ 1pcs, very good</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>800 rmb, little high</t>
+          <t>¥17, Moq 50, good</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>3400, Good price</t>
+          <t>600 RMB Great, very cheap</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>10$</t>
+          <t>800 rmb, little high</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>69$</t>
+          <t>3400, Good price</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>50-85$</t>
+          <t>10$</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2389,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>￥1000 good</t>
+          <t>69$</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>¥ 500 good</t>
+          <t>50-85$</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>￥ 300 good</t>
+          <t>￥1000 good</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>300 rmb and more. Good quality and good price. Small quantity</t>
+          <t>¥ 500 good</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>33$ for 1 pcs. Good quality and quantity</t>
+          <t>￥ 300 good</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
+          <t>300 rmb and more. Good quality and good price. Small quantity</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Good 👍</t>
+          <t>33$ for 1 pcs. Good quality and quantity</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1570</t>
+          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>Good 👍</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>130 yuan | 1410</t>
+          <t>1570</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>20000usd</t>
+          <t>5800</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>500yuan</t>
+          <t>130 yuan</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>MOQ 100, 47 rnb per piece</t>
+          <t>20000usd</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>MOQ 50, 200 rnb per</t>
+          <t>500yuan</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>MOQ 10, 845 per piece | 800usd, very nice, good quality product</t>
+          <t>MOQ 100, 47 rnb per piece</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>1pcs. Start from 60rmb. Novative technology</t>
+          <t>MOQ 50, 200 rnb per</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>From 1pc. Natural materials.</t>
+          <t>MOQ 10, 845 per piece</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>1250rmb. MOQ 1 pc</t>
+          <t>1pcs. Start from 60rmb. Novative technology</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>From 1pc. Natural materials.</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>1410 | 199</t>
+          <t>1250rmb. MOQ 1 pc</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>399</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>199</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>150 yuan, 100, good range of products</t>
+          <t>329</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
+          <t>229</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
+          <t>680</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
+          <t>150 yuan, 100, good range of products</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>I couldn't tell you the price for smart pens right away, but they said they would send a catalogue with prices to Wechat</t>
+          <t>800usd, very nice, good quality product</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
         </is>
       </c>
     </row>
@@ -3490,7 +3490,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
+          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с емкой батареей . Опять же проблема с ПО .</t>
+          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3556,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
+          <t>I couldn't tell you the price for smart pens right away, but they said they would send a catalogue with prices to Wechat</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного метра 150 юаней сказала примерно. Не до </t>
+          <t>199</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
+          <t>320</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t xml:space="preserve">От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккуратно. Хорошее решение для сушки белья и </t>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
         </is>
       </c>
     </row>
@@ -3753,7 +3753,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
+          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с емкой батареей . Опять же проблема с ПО .</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3782,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
+          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>600</t>
+          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного метра 150 юаней сказала примерно. Не до </t>
         </is>
       </c>
     </row>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>43</t>
+          <t xml:space="preserve">От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккуратно. Хорошее решение для сушки белья и </t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>0.6 usd/m2</t>
+          <t>2900 usd</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Under negotiation, great opportunities</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>1-5 usd/l</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>679 rmb</t>
+          <t>MOQ 1, they got samples. 8000usd. Very well made product, trendy and popular. This capsules houses very affordable.</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>59 rmb</t>
+          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>249RMB</t>
+          <t>600</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>6000RMB</t>
+          <t>500</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2000RMB&amp;gt;</t>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>MOQ - 5000 and price - 7000 dollars | 3000 USD | 2147</t>
+          <t>0.6 usd/m2</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>3000 dollars</t>
+          <t>Under negotiation, great opportunities</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>The price cheap, merchant very friendly</t>
+          <t>1-5 usd/l</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>The price more cheaper, good quality</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Good merchant, perfect products</t>
+          <t>679 rmb</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
+          <t>59 rmb</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>15 RMB the product is interesting</t>
+          <t>249RMB</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>nearly $15,000 for this production line</t>
+          <t>6000RMB</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>2000RMB&amp;gt;</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>MOQ - 5000 and price - 7000 dollars</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>5000 USD | 2085 | 2223</t>
+          <t>4000$</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>6000 RMB. I like the way they explain everything about their product.</t>
+          <t>3000 dollars</t>
         </is>
       </c>
     </row>
@@ -4735,7 +4735,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
+          <t>The price cheap, merchant very friendly</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>249 RMB. They have fully described their products. | 249RMB , 价格很便宜</t>
+          <t>The price more cheaper, good quality</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>6000RMB，积极，详细地告诉了一切</t>
+          <t>Good merchant, perfect products</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2000 RMB</t>
+          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>400rmb /m2 good meeting | 400rmb/m2</t>
+          <t>15 RMB the product is interesting</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>350 rmb/m2 | 350rmb/m2</t>
+          <t>nearly $15,000 for this production line</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>20 / MOQ 100 Nice worker answered all questions</t>
+          <t>249</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>80 rmb for 230 meter</t>
+          <t>749</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>1560 rmb for whole item</t>
+          <t>5000 USD</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>4600 rmb</t>
+          <t>3000 USD</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>3000 USD</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>6000 RMB. I like the way they explain everything about their product.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
+          <t>249 RMB. They have fully described their products.</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>250¥/м3 | 250¥/m3</t>
+          <t>6000RMB，积极，详细地告诉了一切</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>4500¥ | 4500¥</t>
+          <t>249RMB , 价格很便宜</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>300¥ 300pcs</t>
+          <t>2000 RMB</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>50¥ 1000pcs</t>
+          <t>400rmb /m2 good meeting</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>500$ 100psc</t>
+          <t>350 rmb/m2</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
+          <t>MOQ 5000 pieces</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
+          <t>400rmb/m2</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
+          <t>350rmb/m2</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
+          <t>MOQ 5000 pieces</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>100 RMB per sample. The taste is very good</t>
+          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>150 RMB per sample. The taste is very good</t>
+          <t>3000 / MOQ 1 Inside view is luxury, i love it</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5677,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>250 RMB per sample. The taste is very good</t>
+          <t>20 / MOQ 100 Nice worker answered all questions</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>498rmb/unit. I like the green tea in white color. First time to see colorless tea and it was amazing, i will recommend i</t>
+          <t>80 rmb for 230 meter</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea. | The 中国好水 brand water w</t>
+          <t>1560 rmb for whole item</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5780,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>4600 rmb</t>
         </is>
       </c>
     </row>
@@ -5821,7 +5821,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Prices are go and packing and Verstaliy is more</t>
+          <t>150 Yuan, 1 bottle. ( Taste is strong and good</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6002,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>The taste anaroma is good of this product then anyother</t>
+          <t>Haven't discussed the prices. Just got the company name list for future reference</t>
         </is>
       </c>
     </row>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>the product prices are very good. looks attractive</t>
+          <t>2085</t>
         </is>
       </c>
     </row>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>650 moq 300</t>
+          <t>2147</t>
         </is>
       </c>
     </row>
@@ -6093,7 +6093,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>560 moq 200</t>
+          <t>2223</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
+          <t>250¥/м3</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
+          <t>4500¥</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>20 | Жду коммерческое предложение. Компания понравилась</t>
+          <t>8790$</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>300¥ 300pcs</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6286,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>9$</t>
+          <t>50¥ 1000pcs</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>13.25$</t>
+          <t>500$ 100psc</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>8.83$</t>
+          <t>4500¥</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>640 PCs, 3.72 RMB very good</t>
+          <t>8790$</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>30 PCs, 420 RMB, need check quality</t>
+          <t>250¥/m3</t>
         </is>
       </c>
     </row>
@@ -6463,7 +6463,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>10 PCs, 1150 RMB, very good</t>
+          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
         </is>
       </c>
     </row>
@@ -6504,7 +6504,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6545,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>1p, 10000$m2, very beautiful big red door</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1 container (400 square meters), 60 dollars for 1 square meters</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Depend on item</t>
+          <t>Moq is 1 door, 530 RMB for 1 door</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Depend of quantity</t>
+          <t>14400 dollars, moq - 1</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>100/square meter</t>
+          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>RMB 15705 MOQ5; pleasant impression</t>
+          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6795,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>MOQ5 25799 RMB</t>
+          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6840,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>RMB 19479; MOQ 1</t>
+          <t>100 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>150 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>250 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -6975,7 +6975,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>498rmb/unit. I like the green tea in white color. First time to see colorless tea and it was amazing, i will recommend i</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>2000$, can be customized, very convenient</t>
+          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea.</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>38$, very unique</t>
+          <t>The 中国好水 brand water was really good. They are using deep water instead of shallow water (used by nongfu), and trace min</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7110,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>2050 rmb, very interesting, convenient to use for pets</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>25 rmb, 1 box, like this product | 1 container 500 rmb</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7188,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>34 rmb, 1000, normal</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>40 rmb, 2000, very good</t>
+          <t>1100</t>
         </is>
       </c>
     </row>
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1 container 250 rmb</t>
+          <t>1050</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Цена зависит от обьема, от 3 юаней, расходники</t>
+          <t>550</t>
         </is>
       </c>
     </row>
@@ -7348,9 +7348,984 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
+          <t>Prices are go and packing and Verstaliy is more</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr"/>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>The taste anaroma is good of this product then anyother</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr"/>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>the product prices are very good. looks attractive</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr"/>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>820 rmb moq 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr"/>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>650 moq 300</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr"/>
+      <c r="C187" t="inlineStr"/>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>560 moq 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr"/>
+      <c r="C188" t="inlineStr"/>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>2.5 RMB per unit, MOQ is 500 pieces. The plastic material was high quality and company was willing to provide samples on</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr"/>
+      <c r="C189" t="inlineStr"/>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr"/>
+      <c r="C190" t="inlineStr"/>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr"/>
+      <c r="C191" t="inlineStr"/>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1299, MOQ 200. I like the company and people there . Very friendly and know their products very good . I would be happy </t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr"/>
+      <c r="C192" t="inlineStr"/>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>5000rmb MOQ 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr"/>
+      <c r="C193" t="inlineStr"/>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>1500 rmb MOQ 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr"/>
+      <c r="C194" t="inlineStr"/>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Black matt tap water $20</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr"/>
+      <c r="C195" t="inlineStr"/>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr"/>
+      <c r="C196" t="inlineStr"/>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr"/>
+      <c r="C197" t="inlineStr"/>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>9$</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr"/>
+      <c r="C198" t="inlineStr"/>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>13.25$</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr"/>
+      <c r="C199" t="inlineStr"/>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>8.83$</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr"/>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>640 PCs, 3.72 RMB very good</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr"/>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>30 PCs, 420 RMB, need check quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr"/>
+      <c r="C202" t="inlineStr"/>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>10 PCs, 1150 RMB, very good</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr"/>
+      <c r="C203" t="inlineStr"/>
+      <c r="D203" t="inlineStr"/>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr"/>
+      <c r="C204" t="inlineStr"/>
+      <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr"/>
+      <c r="C205" t="inlineStr"/>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr"/>
+      <c r="C206" t="inlineStr"/>
+      <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Depend on item</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr"/>
+      <c r="C207" t="inlineStr"/>
+      <c r="D207" t="inlineStr"/>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr"/>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Depend of quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr"/>
+      <c r="C208" t="inlineStr"/>
+      <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr"/>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>100/square meter</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr"/>
+      <c r="C209" t="inlineStr"/>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr"/>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>RMB 15705 MOQ5; pleasant impression</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr"/>
+      <c r="C210" t="inlineStr"/>
+      <c r="D210" t="inlineStr"/>
+      <c r="E210" t="inlineStr"/>
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="inlineStr"/>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>MOQ5 25799 RMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr"/>
+      <c r="C211" t="inlineStr"/>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr"/>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>RMB 19479; MOQ 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr"/>
+      <c r="C212" t="inlineStr"/>
+      <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr"/>
+      <c r="G212" t="inlineStr"/>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr"/>
+      <c r="C213" t="inlineStr"/>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr"/>
+      <c r="C214" t="inlineStr"/>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr"/>
+      <c r="C215" t="inlineStr"/>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>2000$, can be customized, very convenient</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr"/>
+      <c r="C216" t="inlineStr"/>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>38$, very unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr"/>
+      <c r="C217" t="inlineStr"/>
+      <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>2050 rmb, very interesting, convenient to use for pets</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr"/>
+      <c r="C218" t="inlineStr"/>
+      <c r="D218" t="inlineStr"/>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>25 rmb, 1 box, like this product</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr"/>
+      <c r="C219" t="inlineStr"/>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>34 rmb, 1000, normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr"/>
+      <c r="C220" t="inlineStr"/>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>40 rmb, 2000, very good</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr"/>
+      <c r="C221" t="inlineStr"/>
+      <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>1 container 250 rmb</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr"/>
+      <c r="C222" t="inlineStr"/>
+      <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>1 container 500 rmb</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr"/>
+      <c r="C223" t="inlineStr"/>
+      <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>1 container 700 rmb</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr"/>
+      <c r="C224" t="inlineStr"/>
+      <c r="D224" t="inlineStr"/>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Жду коммерческое предложение. Компания понравилась</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr"/>
+      <c r="C225" t="inlineStr"/>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Цена зависит от обьема, от 3 юаней, расходники</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr"/>
+      <c r="C226" t="inlineStr"/>
+      <c r="D226" t="inlineStr"/>
+      <c r="E226" t="inlineStr"/>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
           <t>Прайс отправят, от 100ед, хорошая компания</t>
         </is>
       </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr"/>
+      <c r="C227" t="inlineStr"/>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr"/>
+      <c r="C228" t="inlineStr"/>
+      <c r="D228" t="inlineStr"/>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr"/>
+      <c r="C229" t="inlineStr"/>
+      <c r="D229" t="inlineStr"/>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
CBD: fix 1:1 card-product, proper OCR mapping
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I229"/>
+  <dimension ref="A1:I183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,11 +590,7 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Supplier_Row3_1</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
@@ -647,7 +643,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -836,7 +832,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -861,7 +857,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1046,7 +1042,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1132,7 +1128,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1145,11 +1141,7 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Supplier_Row8_1</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
@@ -1444,7 +1436,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1530,7 +1522,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1575,7 +1567,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1657,7 +1649,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Furniture</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1739,7 +1731,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Furniture</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1995,7 +1987,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>620 super</t>
+          <t>130 super</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2028,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1500 super</t>
+          <t>$32, MOQ 300, good</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2073,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>130 super</t>
+          <t>¥3000, MoQ 1pcs, very good</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2118,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>$32, MOQ 300, good</t>
+          <t>¥17, Moq 50, good</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2163,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>¥3000, MoQ 1pcs, very good</t>
+          <t>600 RMB Great, very cheap</t>
         </is>
       </c>
     </row>
@@ -2179,11 +2171,7 @@
       <c r="A46" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Supplier_Row17_2</t>
-        </is>
-      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
@@ -2196,7 +2184,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>¥17, Moq 50, good</t>
+          <t>800 rmb, little high</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2213,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>600 RMB Great, very cheap</t>
+          <t>3400, Good price</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2254,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>800 rmb, little high</t>
+          <t>10$</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2299,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3400, Good price</t>
+          <t>69$</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2340,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>10$</t>
+          <t>50-85$</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2377,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>69$</t>
+          <t>￥1000 good</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2422,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>50-85$</t>
+          <t>¥ 500 good</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2467,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>￥1000 good</t>
+          <t>￥ 300 good</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2500,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>¥ 500 good</t>
+          <t>300 rmb and more. Good quality and good price. Small quantity</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2545,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>￥ 300 good</t>
+          <t>33$ for 1 pcs. Good quality and quantity</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2578,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>300 rmb and more. Good quality and good price. Small quantity</t>
+          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2611,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>33$ for 1 pcs. Good quality and quantity</t>
+          <t>Good 👍</t>
         </is>
       </c>
     </row>
@@ -2631,11 +2619,7 @@
       <c r="A58" t="n">
         <v>57</v>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Supplier_Row21_2</t>
-        </is>
-      </c>
+      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
@@ -2648,7 +2632,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Good quality and quantity. 140 rmb 1 pcs.</t>
+          <t>1570</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2677,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Good 👍</t>
+          <t>5800</t>
         </is>
       </c>
     </row>
@@ -2733,12 +2717,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>1570</t>
+          <t>130 yuan</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2767,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>20000usd</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2812,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>130 yuan</t>
+          <t>500yuan</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2857,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>20000usd</t>
+          <t>MOQ 100, 47 rnb per piece</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2898,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>500yuan</t>
+          <t>MOQ 50, 200 rnb per</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2938,12 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>MOQ 100, 47 rnb per piece</t>
+          <t>MOQ 10, 845 per piece</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2983,12 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>MOQ 50, 200 rnb per</t>
+          <t>1pcs. Start from 60rmb. Novative technology</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3013,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>MOQ 10, 845 per piece</t>
+          <t>From 1pc. Natural materials.</t>
         </is>
       </c>
     </row>
@@ -3049,12 +3033,12 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>1pcs. Start from 60rmb. Novative technology</t>
+          <t>1250rmb. MOQ 1 pc</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3058,12 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>From 1pc. Natural materials.</t>
+          <t>199</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3104,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>1250rmb. MOQ 1 pc</t>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3144,12 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>329</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3190,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>229</t>
         </is>
       </c>
     </row>
@@ -3238,12 +3222,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>680</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3272,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>150 yuan, 100, good range of products</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3312,12 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3342,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
         </is>
       </c>
     </row>
@@ -3394,12 +3378,12 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>150 yuan, 100, good range of products</t>
+          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
         </is>
       </c>
     </row>
@@ -3407,11 +3391,7 @@
       <c r="A78" t="n">
         <v>77</v>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Supplier_Row28_3</t>
-        </is>
-      </c>
+      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
@@ -3419,12 +3399,12 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>800usd, very nice, good quality product</t>
+          <t>I couldn't tell you the price for smart pens right away, but they said they would send a catalogue with prices to Wechat</t>
         </is>
       </c>
     </row>
@@ -3432,11 +3412,7 @@
       <c r="A79" t="n">
         <v>78</v>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Supplier_Row29_2</t>
-        </is>
-      </c>
+      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
@@ -3449,7 +3425,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
+          <t>320</t>
         </is>
       </c>
     </row>
@@ -3485,12 +3461,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
+          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
         </is>
       </c>
     </row>
@@ -3498,11 +3474,7 @@
       <c r="A81" t="n">
         <v>80</v>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Supplier_Row30_2</t>
-        </is>
-      </c>
+      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
@@ -3515,7 +3487,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
+          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с емкой батареей . Опять же проблема с ПО .</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3528,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>I couldn't tell you the price for smart pens right away, but they said they would send a catalogue with prices to Wechat</t>
+          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3573,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>199</t>
+          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного метра 150 юаней сказала примерно. Не до </t>
         </is>
       </c>
     </row>
@@ -3638,7 +3610,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3635,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t xml:space="preserve">От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккуратно. Хорошее решение для сушки белья и </t>
         </is>
       </c>
     </row>
@@ -3708,7 +3680,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -3753,7 +3725,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>330 юаней. 500 штук минималка . Качественный , магнитный умный переключатель с емкой батареей . Опять же проблема с ПО .</t>
+          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
         </is>
       </c>
     </row>
@@ -3761,11 +3733,7 @@
       <c r="A88" t="n">
         <v>87</v>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Supplier_Row33_3</t>
-        </is>
-      </c>
+      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
@@ -3782,7 +3750,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
+          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3795,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Необычный вариант стены. Можно очень вариативно украсить. Стоимость квадратного метра 150 юаней сказала примерно. Не до </t>
+          <t>600</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3820,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
+          <t>500</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3845,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t xml:space="preserve">От одной закути. Видела и раньше такие конструкции, но эти выглядели очень аккуратно. Хорошее решение для сушки белья и </t>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3890,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2900 usd</t>
+          <t>0.6 usd/m2</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3935,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Under negotiation, great opportunities</t>
         </is>
       </c>
     </row>
@@ -4004,7 +3972,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1-5 usd/l</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4005,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4030,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>MOQ 1, they got samples. 8000usd. Very well made product, trendy and popular. This capsules houses very affordable.</t>
+          <t>679 rmb</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4059,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
+          <t>59 rmb</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4088,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>249RMB</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4129,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>6000RMB</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4162,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>2000RMB&amp;gt;</t>
         </is>
       </c>
     </row>
@@ -4230,12 +4198,12 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>0.6 usd/m2</t>
+          <t>MOQ - 5000 and price - 7000 dollars</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4248,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Under negotiation, great opportunities</t>
+          <t>3000 dollars</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4289,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>1-5 usd/l</t>
+          <t>The price cheap, merchant very friendly</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4330,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>The price more cheaper, good quality</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4375,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>679 rmb</t>
+          <t>Good merchant, perfect products</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4420,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>59 rmb</t>
+          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4465,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>249RMB</t>
+          <t>15 RMB the product is interesting</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4510,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>6000RMB</t>
+          <t>nearly $15,000 for this production line</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4555,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2000RMB&amp;gt;</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4596,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>MOQ - 5000 and price - 7000 dollars</t>
+          <t>749</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4641,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>4000$</t>
+          <t>5000 USD</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4670,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>3000 dollars</t>
+          <t>6000 RMB. I like the way they explain everything about their product.</t>
         </is>
       </c>
     </row>
@@ -4730,12 +4698,12 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>The price cheap, merchant very friendly</t>
+          <t>Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
         </is>
       </c>
     </row>
@@ -4763,12 +4731,12 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>The price more cheaper, good quality</t>
+          <t>249 RMB. They have fully described their products.</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4769,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Good merchant, perfect products</t>
+          <t>6000RMB，积极，详细地告诉了一切</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4798,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
+          <t>2000 RMB</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4839,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>15 RMB the product is interesting</t>
+          <t>400rmb /m2 good meeting</t>
         </is>
       </c>
     </row>
@@ -4903,12 +4871,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Furniture &amp; Custom Home</t>
+          <t>Furniture</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>nearly $15,000 for this production line</t>
+          <t>350 rmb/m2</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4921,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
         </is>
       </c>
     </row>
@@ -4989,12 +4957,12 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>20 / MOQ 100 Nice worker answered all questions</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5003,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>80 rmb for 230 meter</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5044,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>5000 USD</t>
+          <t>1560 rmb for whole item</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5089,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>3000 USD</t>
+          <t>4600 rmb</t>
         </is>
       </c>
     </row>
@@ -5129,11 +5097,7 @@
       <c r="A124" t="n">
         <v>123</v>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Supplier_Row49_1</t>
-        </is>
-      </c>
+      <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr"/>
@@ -5146,7 +5110,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>3000 USD</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5154,11 +5118,7 @@
       <c r="A125" t="n">
         <v>124</v>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Supplier_Row49_2</t>
-        </is>
-      </c>
+      <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
@@ -5171,7 +5131,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>6000 RMB. I like the way they explain everything about their product.</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5179,11 +5139,7 @@
       <c r="A126" t="n">
         <v>125</v>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Supplier_Row49_3</t>
-        </is>
-      </c>
+      <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
@@ -5196,7 +5152,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5177,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>249 RMB. They have fully described their products.</t>
+          <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5218,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>6000RMB，积极，详细地告诉了一切</t>
+          <t>250¥/м3</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5263,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>249RMB , 价格很便宜</t>
+          <t>4500¥</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5308,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2000 RMB</t>
+          <t>300¥ 300pcs</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5349,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>400rmb /m2 good meeting</t>
+          <t>50¥ 1000pcs</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5394,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>350 rmb/m2</t>
+          <t>500$ 100psc</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5435,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>MOQ 5000 pieces</t>
+          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
         </is>
       </c>
     </row>
@@ -5519,12 +5475,12 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>400rmb/m2</t>
+          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5509,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>350rmb/m2</t>
+          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5534,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>MOQ 5000 pieces</t>
+          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5571,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
+          <t>100 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5608,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>3000 / MOQ 1 Inside view is luxury, i love it</t>
+          <t>150 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5633,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>20 / MOQ 100 Nice worker answered all questions</t>
+          <t>250 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5658,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>80 rmb for 230 meter</t>
+          <t>498rmb/unit. I like the green tea in white color. First time to see colorless tea and it was amazing, i will recommend i</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5691,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>1560 rmb for whole item</t>
+          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea.</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5736,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>4600 rmb</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -5821,7 +5777,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5818,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5863,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>1100</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5908,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>50 Yuan 50g (The taste is authentic and aroma is really good</t>
+          <t>1050</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5933,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>150 Yuan, 1 bottle. ( Taste is strong and good</t>
+          <t>Prices are go and packing and Verstaliy is more</t>
         </is>
       </c>
     </row>
@@ -6002,7 +5958,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Haven't discussed the prices. Just got the company name list for future reference</t>
+          <t>The taste anaroma is good of this product then anyother</t>
         </is>
       </c>
     </row>
@@ -6027,7 +5983,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2085</t>
+          <t>the product prices are very good. looks attractive</t>
         </is>
       </c>
     </row>
@@ -6068,7 +6024,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2147</t>
+          <t>650 moq 300</t>
         </is>
       </c>
     </row>
@@ -6076,11 +6032,7 @@
       <c r="A151" t="n">
         <v>150</v>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Supplier_Row63_3</t>
-        </is>
-      </c>
+      <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr"/>
@@ -6093,7 +6045,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>560 moq 200</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6086,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>250¥/м3</t>
+          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6123,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>4500¥</t>
+          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6168,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>8790$</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6224,11 +6176,7 @@
       <c r="A155" t="n">
         <v>154</v>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Supplier_Row66_3</t>
-        </is>
-      </c>
+      <c r="B155" t="inlineStr"/>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr"/>
@@ -6241,7 +6189,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>300¥ 300pcs</t>
+          <t>109</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6234,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>50¥ 1000pcs</t>
+          <t>9$</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6271,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>500$ 100psc</t>
+          <t>13.25$</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6312,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>4500¥</t>
+          <t>8.83$</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6345,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>8790$</t>
+          <t>640 PCs, 3.72 RMB very good</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6386,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>250¥/m3</t>
+          <t>30 PCs, 420 RMB, need check quality</t>
         </is>
       </c>
     </row>
@@ -6446,11 +6394,7 @@
       <c r="A161" t="n">
         <v>160</v>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Supplier_Row68_3</t>
-        </is>
-      </c>
+      <c r="B161" t="inlineStr"/>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr"/>
@@ -6463,7 +6407,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
+          <t>10 PCs, 1150 RMB, very good</t>
         </is>
       </c>
     </row>
@@ -6499,12 +6443,12 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6489,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>1p, 10000$m2, very beautiful big red door</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6530,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>1 container (400 square meters), 60 dollars for 1 square meters</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -6626,12 +6570,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Moq is 1 door, 530 RMB for 1 door</t>
+          <t>Depend on item</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6604,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>14400 dollars, moq - 1</t>
+          <t>Depend of quantity</t>
         </is>
       </c>
     </row>
@@ -6700,12 +6644,12 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Smart Home</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
+          <t>100/square meter</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6694,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
+          <t>RMB 15705 MOQ5; pleasant impression</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6739,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Индивидуальный от размеров. Нет уен конкретных у всех поставщиков. Все делается под заказ и производится от 1 шт.</t>
+          <t>MOQ5 25799 RMB</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6784,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>100 RMB per sample. The taste is very good</t>
+          <t>RMB 19479; MOQ 1</t>
         </is>
       </c>
     </row>
@@ -6880,12 +6824,12 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>150 RMB per sample. The taste is very good</t>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6874,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>250 RMB per sample. The taste is very good</t>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -6970,12 +6914,12 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>498rmb/unit. I like the green tea in white color. First time to see colorless tea and it was amazing, i will recommend i</t>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -7020,7 +6964,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea.</t>
+          <t>2000$, can be customized, very convenient</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7009,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>The 中国好水 brand water was really good. They are using deep water instead of shallow water (used by nongfu), and trace min</t>
+          <t>38$, very unique</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7054,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>2050 rmb, very interesting, convenient to use for pets</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7087,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>25 rmb, 1 box, like this product</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7132,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>34 rmb, 1000, normal</t>
         </is>
       </c>
     </row>
@@ -7228,12 +7172,12 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>40 rmb, 2000, very good</t>
         </is>
       </c>
     </row>
@@ -7278,7 +7222,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1 container 250 rmb</t>
         </is>
       </c>
     </row>
@@ -7288,32 +7232,32 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>ZHEJIANG TIANYAN HOLDING CO.,LTD.</t>
+          <t>宏宇集团 HONGYU GROUP</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Nicole</t>
+          <t>Melina 王玲</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ty11@cntianyan.com</t>
+          <t>lina@hongyugroup.com</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>+86-15867028552</t>
+          <t>+86 13827702216</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>www.cntianyan.com</t>
+          <t>en.hongyugroup.com</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Chengjiang industrial zone,huangyan district taizhou,zhejiang,china</t>
+          <t>广东省佛山市禅城区江湾二路26号 (No.26 Jiangwan Second Road, Chancheng District, Foshan, Guangdong)</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -7323,7 +7267,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>Жду коммерческое предложение. Компания понравилась</t>
         </is>
       </c>
     </row>
@@ -7333,14 +7277,34 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>BANRUGE / KING LIYE</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr"/>
-      <c r="D182" t="inlineStr"/>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr"/>
+          <t>ZHEJIANG TIANYAN HOLDING CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>ty11@cntianyan.com</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>+86-15867028552</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>www.cntianyan.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Chengjiang industrial zone,huangyan district taizhou,zhejiang,china</t>
+        </is>
+      </c>
       <c r="H182" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -7348,7 +7312,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Prices are go and packing and Verstaliy is more</t>
+          <t>Цена зависит от обьема, от 3 юаней, расходники</t>
         </is>
       </c>
     </row>
@@ -7356,7 +7320,11 @@
       <c r="A183" t="n">
         <v>182</v>
       </c>
-      <c r="B183" t="inlineStr"/>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>BANRUGE / KING LIYE</t>
+        </is>
+      </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr"/>
@@ -7364,968 +7332,14 @@
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Building Decoration</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>The taste anaroma is good of this product then anyother</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
-        <v>183</v>
-      </c>
-      <c r="B184" t="inlineStr"/>
-      <c r="C184" t="inlineStr"/>
-      <c r="D184" t="inlineStr"/>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>the product prices are very good. looks attractive</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="n">
-        <v>184</v>
-      </c>
-      <c r="B185" t="inlineStr"/>
-      <c r="C185" t="inlineStr"/>
-      <c r="D185" t="inlineStr"/>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>820 rmb moq 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="n">
-        <v>185</v>
-      </c>
-      <c r="B186" t="inlineStr"/>
-      <c r="C186" t="inlineStr"/>
-      <c r="D186" t="inlineStr"/>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>650 moq 300</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="n">
-        <v>186</v>
-      </c>
-      <c r="B187" t="inlineStr"/>
-      <c r="C187" t="inlineStr"/>
-      <c r="D187" t="inlineStr"/>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>560 moq 200</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="n">
-        <v>187</v>
-      </c>
-      <c r="B188" t="inlineStr"/>
-      <c r="C188" t="inlineStr"/>
-      <c r="D188" t="inlineStr"/>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>2.5 RMB per unit, MOQ is 500 pieces. The plastic material was high quality and company was willing to provide samples on</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>188</v>
-      </c>
-      <c r="B189" t="inlineStr"/>
-      <c r="C189" t="inlineStr"/>
-      <c r="D189" t="inlineStr"/>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr"/>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="n">
-        <v>189</v>
-      </c>
-      <c r="B190" t="inlineStr"/>
-      <c r="C190" t="inlineStr"/>
-      <c r="D190" t="inlineStr"/>
-      <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr"/>
-      <c r="G190" t="inlineStr"/>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="n">
-        <v>190</v>
-      </c>
-      <c r="B191" t="inlineStr"/>
-      <c r="C191" t="inlineStr"/>
-      <c r="D191" t="inlineStr"/>
-      <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr"/>
-      <c r="G191" t="inlineStr"/>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1299, MOQ 200. I like the company and people there . Very friendly and know their products very good . I would be happy </t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="n">
-        <v>191</v>
-      </c>
-      <c r="B192" t="inlineStr"/>
-      <c r="C192" t="inlineStr"/>
-      <c r="D192" t="inlineStr"/>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>5000rmb MOQ 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="n">
-        <v>192</v>
-      </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>1500 rmb MOQ 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="n">
-        <v>193</v>
-      </c>
-      <c r="B194" t="inlineStr"/>
-      <c r="C194" t="inlineStr"/>
-      <c r="D194" t="inlineStr"/>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr"/>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>Black matt tap water $20</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>194</v>
-      </c>
-      <c r="B195" t="inlineStr"/>
-      <c r="C195" t="inlineStr"/>
-      <c r="D195" t="inlineStr"/>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
-      <c r="G195" t="inlineStr"/>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="n">
-        <v>195</v>
-      </c>
-      <c r="B196" t="inlineStr"/>
-      <c r="C196" t="inlineStr"/>
-      <c r="D196" t="inlineStr"/>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr"/>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>109</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="n">
-        <v>196</v>
-      </c>
-      <c r="B197" t="inlineStr"/>
-      <c r="C197" t="inlineStr"/>
-      <c r="D197" t="inlineStr"/>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
-      <c r="G197" t="inlineStr"/>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>9$</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>197</v>
-      </c>
-      <c r="B198" t="inlineStr"/>
-      <c r="C198" t="inlineStr"/>
-      <c r="D198" t="inlineStr"/>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>13.25$</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="n">
-        <v>198</v>
-      </c>
-      <c r="B199" t="inlineStr"/>
-      <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>8.83$</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="n">
-        <v>199</v>
-      </c>
-      <c r="B200" t="inlineStr"/>
-      <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>640 PCs, 3.72 RMB very good</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="n">
-        <v>200</v>
-      </c>
-      <c r="B201" t="inlineStr"/>
-      <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr"/>
-      <c r="H201" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>30 PCs, 420 RMB, need check quality</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="n">
-        <v>201</v>
-      </c>
-      <c r="B202" t="inlineStr"/>
-      <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I202" t="inlineStr">
-        <is>
-          <t>10 PCs, 1150 RMB, very good</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="n">
-        <v>202</v>
-      </c>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
-      <c r="H203" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="n">
-        <v>203</v>
-      </c>
-      <c r="B204" t="inlineStr"/>
-      <c r="C204" t="inlineStr"/>
-      <c r="D204" t="inlineStr"/>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="n">
-        <v>204</v>
-      </c>
-      <c r="B205" t="inlineStr"/>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="n">
-        <v>205</v>
-      </c>
-      <c r="B206" t="inlineStr"/>
-      <c r="C206" t="inlineStr"/>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>Depend on item</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="n">
-        <v>206</v>
-      </c>
-      <c r="B207" t="inlineStr"/>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>Depend of quantity</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="n">
-        <v>207</v>
-      </c>
-      <c r="B208" t="inlineStr"/>
-      <c r="C208" t="inlineStr"/>
-      <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>100/square meter</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
-        <v>208</v>
-      </c>
-      <c r="B209" t="inlineStr"/>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr"/>
-      <c r="H209" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t>RMB 15705 MOQ5; pleasant impression</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
-        <v>209</v>
-      </c>
-      <c r="B210" t="inlineStr"/>
-      <c r="C210" t="inlineStr"/>
-      <c r="D210" t="inlineStr"/>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr"/>
-      <c r="H210" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>MOQ5 25799 RMB</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>210</v>
-      </c>
-      <c r="B211" t="inlineStr"/>
-      <c r="C211" t="inlineStr"/>
-      <c r="D211" t="inlineStr"/>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>RMB 19479; MOQ 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>211</v>
-      </c>
-      <c r="B212" t="inlineStr"/>
-      <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>212</v>
-      </c>
-      <c r="B213" t="inlineStr"/>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="n">
-        <v>213</v>
-      </c>
-      <c r="B214" t="inlineStr"/>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="n">
-        <v>214</v>
-      </c>
-      <c r="B215" t="inlineStr"/>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>2000$, can be customized, very convenient</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>215</v>
-      </c>
-      <c r="B216" t="inlineStr"/>
-      <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>38$, very unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="n">
-        <v>216</v>
-      </c>
-      <c r="B217" t="inlineStr"/>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr"/>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
-      <c r="G217" t="inlineStr"/>
-      <c r="H217" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I217" t="inlineStr">
-        <is>
-          <t>2050 rmb, very interesting, convenient to use for pets</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="n">
-        <v>217</v>
-      </c>
-      <c r="B218" t="inlineStr"/>
-      <c r="C218" t="inlineStr"/>
-      <c r="D218" t="inlineStr"/>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
-      <c r="G218" t="inlineStr"/>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I218" t="inlineStr">
-        <is>
-          <t>25 rmb, 1 box, like this product</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>218</v>
-      </c>
-      <c r="B219" t="inlineStr"/>
-      <c r="C219" t="inlineStr"/>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr">
-        <is>
-          <t>34 rmb, 1000, normal</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
-        <v>219</v>
-      </c>
-      <c r="B220" t="inlineStr"/>
-      <c r="C220" t="inlineStr"/>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I220" t="inlineStr">
-        <is>
-          <t>40 rmb, 2000, very good</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>220</v>
-      </c>
-      <c r="B221" t="inlineStr"/>
-      <c r="C221" t="inlineStr"/>
-      <c r="D221" t="inlineStr"/>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
-      <c r="G221" t="inlineStr"/>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I221" t="inlineStr">
-        <is>
-          <t>1 container 250 rmb</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>221</v>
-      </c>
-      <c r="B222" t="inlineStr"/>
-      <c r="C222" t="inlineStr"/>
-      <c r="D222" t="inlineStr"/>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr"/>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I222" t="inlineStr">
-        <is>
-          <t>1 container 500 rmb</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>222</v>
-      </c>
-      <c r="B223" t="inlineStr"/>
-      <c r="C223" t="inlineStr"/>
-      <c r="D223" t="inlineStr"/>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
-      <c r="G223" t="inlineStr"/>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I223" t="inlineStr">
-        <is>
-          <t>1 container 700 rmb</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>223</v>
-      </c>
-      <c r="B224" t="inlineStr"/>
-      <c r="C224" t="inlineStr"/>
-      <c r="D224" t="inlineStr"/>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr"/>
-      <c r="H224" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I224" t="inlineStr">
-        <is>
-          <t>Жду коммерческое предложение. Компания понравилась</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="n">
-        <v>224</v>
-      </c>
-      <c r="B225" t="inlineStr"/>
-      <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I225" t="inlineStr">
-        <is>
-          <t>Цена зависит от обьема, от 3 юаней, расходники</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
-        <v>225</v>
-      </c>
-      <c r="B226" t="inlineStr"/>
-      <c r="C226" t="inlineStr"/>
-      <c r="D226" t="inlineStr"/>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
-      <c r="G226" t="inlineStr"/>
-      <c r="H226" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I226" t="inlineStr">
-        <is>
           <t>Прайс отправят, от 100ед, хорошая компания</t>
         </is>
       </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
-        <v>226</v>
-      </c>
-      <c r="B227" t="inlineStr"/>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr"/>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I227" t="inlineStr"/>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
-        <v>227</v>
-      </c>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I228" t="inlineStr"/>
-    </row>
-    <row r="229">
-      <c r="A229" t="n">
-        <v>228</v>
-      </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
-      <c r="H229" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I229" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
CBD: fix categories translated to Russian
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -567,14 +567,11 @@
           <t>张硕怡 (Stoney)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>134 1416 0636</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Doors &amp; Windows</t>
@@ -750,7 +747,6 @@
           <t>WWW.DEIOUXWINDOWS.COM / WWW.DEIOUX-WINDOW.COM</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Doors &amp; Windows</t>
@@ -771,7 +767,6 @@
           <t>China Warren Windows and Doors Co., Ltd.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>info@warrenwindows.com</t>
@@ -839,7 +834,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -877,7 +872,6 @@
           <t>www.hdlautomation.com</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -948,13 +942,11 @@
           <t>邹隆鹏</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>15818099349</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>佛山市顺德区北滘镇顺江社区兴业东路2号启德置业园5栋1楼 (1st Floor, Building 5, Qide Real Estate Park, No. 2 Xingye East Road, Shunjiang, Beijiao Town, Shunde District, Foshan City)</t>
@@ -1040,7 +1032,6 @@
           <t>0086-182 5765 3405, 0086-576-87493988</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Xuanmen Industrial Zone, Yuhuan, Zhejiang, China, 317608</t>
@@ -1071,13 +1062,11 @@
           <t>王小忠</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>189 6909 8963, 0571-8936 7998, 89367999, 180 7280 6350, 300 755 1089</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>浙江省杭州市临平区运河街道育士路53-1号</t>
@@ -1163,7 +1152,6 @@
           <t>13326792105</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>广东省佛山市南海区狮山镇博爱东路博爱工业区横跨路一号(2号厂房)</t>
@@ -1171,7 +1159,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1204,7 +1192,6 @@
           <t>+86-18906831082</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Jiaxing/Hongkong</t>
@@ -1245,7 +1232,6 @@
           <t>+86-18302200384</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Shijiazhuang City, Hebei Province</t>
@@ -1343,7 +1329,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1388,7 +1374,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1411,13 +1397,11 @@
           <t>赖华芳</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>13727479513, 400-8339513</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>广东省佛山市顺德区龙江镇联塑嘉园三路3号9513家具总部</t>
@@ -1463,7 +1447,6 @@
           <t>www.guhaogroup.com / www.cqsdmy.com</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -1499,7 +1482,6 @@
           <t>159 1909 0393, +86-757-2339 1505</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>广东省佛山市顺德区乐从镇黎湖工业区</t>
@@ -1552,7 +1534,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1597,7 +1579,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Doors &amp; Windows</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1620,13 +1602,11 @@
           <t>罗美玲</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>180 0760 4399</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>广东省中山市小榄镇东升门业生产基地F5B</t>
@@ -1634,7 +1614,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1697,15 +1677,11 @@
           <t>超友皮革家居</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>1561767</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -1741,7 +1717,6 @@
           <t>+86-13392758223</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>广东省佛山市顺德区均安镇智安北路12号 (No.12 Zhi'an North Road, Jun'an, Shunde, Foshan, Guangdong, China)</t>
@@ -1749,7 +1724,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1794,7 +1769,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1839,7 +1814,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1902,7 +1877,6 @@
           <t>常州市永春保温材料有限公司 (Changzhou Yongchun Thermal Insulation Materials Co., Ltd.)</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>yc@ycbycl.com</t>
@@ -1993,7 +1967,6 @@
           <t>唐佳豪 (Vance)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>+86 18925924350</t>
@@ -2044,8 +2017,6 @@
           <t>+86 13556688832</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -2156,14 +2127,11 @@
           <t>江门市新阳刚智能科技有限公司</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>135 3666 7789, 400-9090-518</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>广东省江门市新会区大泽镇万洋众创城38-1号</t>
@@ -2234,7 +2202,6 @@
           <t>三强地毯</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>hengsheng_carpet@163.com</t>
@@ -2245,8 +2212,6 @@
           <t>0769-89807692</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -2339,7 +2304,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2429,7 +2394,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Doors &amp; Windows</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2474,7 +2439,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Bath &amp; Sanitary</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2507,7 +2472,6 @@
           <t>13914649982, 18951488133</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>江苏省盐城市亭湖区青墩头灶工业园全创路十号</t>
@@ -2643,10 +2607,9 @@
           <t>www.jnodwater.com</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2691,7 +2654,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2724,7 +2687,6 @@
           <t>+86 18028330648, +86 18022073939</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>2nd Yongyi Industrial Area, Donghai 5th Road, Dongfeng Town, Zhongshan, Guangdong, China</t>
@@ -2732,7 +2694,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2755,13 +2717,11 @@
           <t>潘禹</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>13691864691</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>广东省惠州市惠城区演达大道19号国安居6楼</t>
@@ -2814,7 +2774,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2897,10 +2857,9 @@
           <t>WWW.HOPSOONER.COM</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2918,7 +2877,6 @@
           <t>视威电子科技（上海）有限公司</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>service@3weitech.com</t>
@@ -2979,7 +2937,6 @@
           <t>www.asnug.com</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -3015,8 +2972,6 @@
           <t>+86 137 6339 3059</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -3122,19 +3077,14 @@
       <c r="A65" t="n">
         <v>64</v>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>15916159866</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3224,7 +3174,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3292,13 +3242,11 @@
           <t>曹双林 (Edith Cao)</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>13286132534, 400-0750-889</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>广东省江门市蓬江区迎宾大道西23号之129</t>
@@ -3339,7 +3287,6 @@
           <t>15915974406</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>广东省广州市番禺区正营创意园2栋二楼 (Second floor, Building 2, Zhengying Creative Park, Panyu District, Guangzhou City, Guangdong Province)</t>
@@ -3347,7 +3294,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Doors &amp; Windows</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3365,14 +3312,11 @@
           <t>双龙智科</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>138 6227 5829, 138 6227 4458, 0512-5666 6666</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>江苏省太仓市双凤镇陆江路1号</t>
@@ -3413,7 +3357,6 @@
           <t>189-2984-9818, 0758-8578545</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>Auto Parts Industrial Park, Jinli Town, Gaoyao District, Zhaoqing, Guangdong</t>
@@ -3421,7 +3364,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3454,7 +3397,6 @@
           <t>+86 134 3318 1558, 0757-8560 9159</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>中国广东省佛山市南海区里水镇大步工业区13号 (No. 13, Dabu Industrial Zone, Lishui Town, Nanhai District, Foshan City, Guangdong Province, China)</t>
@@ -3480,7 +3422,6 @@
           <t>Countermast Technology (Dalian) Company Limited</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>sales.countermast.china@countermast.com</t>
@@ -3683,7 +3624,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3728,7 +3669,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3751,7 +3692,6 @@
           <t>袁佳磊</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>18652449601</t>
@@ -3769,7 +3709,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3832,14 +3772,11 @@
           <t>双龙中科</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>138 6227 5829 / 138 6227 4458 / 0512-5666 6666</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>江苏省太仓市双凤镇陆江路1号</t>
@@ -3865,14 +3802,11 @@
           <t>深圳市家为安智能科技有限公司</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>186-0205-8898 / 400-608-0098</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>广东省佛山市南海区里水镇</t>
@@ -3880,7 +3814,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -3898,9 +3832,6 @@
           <t>广州市优品声学科技有限公司</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>www.gzypsx.com</t>
@@ -3913,7 +3844,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Doors &amp; Windows</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3946,7 +3877,6 @@
           <t>133 9983 5678</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>贵州省赤水市成渝(赤水)家具产业园A3-2</t>
@@ -3977,13 +3907,11 @@
           <t>高学梅</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>17687627315</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>广西南宁邕武路增创工业园区 (Zengchuang Ind Park, Yongwu Rd, Nanning, Guangxi, China)</t>
@@ -4069,7 +3997,6 @@
           <t>+86 178-5768-8782</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>Room 1101, Building A2,2-150# Yunlian Road, Yuhang District, Hangzhou, Zhejiang, PRC 311121</t>
@@ -4077,7 +4004,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Smart Home &amp; Lighting</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4115,7 +4042,6 @@
           <t>https://www.amerdecor.com/</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -4141,7 +4067,6 @@
           <t>王冠</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>+86 13229297183</t>
@@ -4204,7 +4129,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Bath &amp; Sanitary</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4227,7 +4152,6 @@
           <t>朱支群</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>13763963598</t>
@@ -4368,7 +4292,6 @@
           <t>(86) 158 8931 1832</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>3rd Floor, Building C, Golden Apple Innovation Park, Ganli 2nd Road, Longgang District, Shenzhen, 518112, China</t>
@@ -4454,7 +4377,6 @@
           <t>18128752879</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>佛山狮山镇谭边工业区崩岗头路四号之一</t>
@@ -4507,7 +4429,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Doors &amp; Windows</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4530,13 +4452,11 @@
           <t>徐云霞</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>13697981203</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>店面地址：江西省景德镇市国贸广场国贸街1号；厂址：吕蒙高新工业园沟上008号</t>
@@ -4562,8 +4482,6 @@
           <t>苏州东山茶厂 (Suzhou Dongshan Biluochun Tea Co., Ltd.)</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>0512-66281146</t>
@@ -4599,14 +4517,11 @@
           <t>知和香馆</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>15926183211</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>福建永春达埔</t>
@@ -4697,7 +4612,6 @@
           <t>www.ptat.cn</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -4723,7 +4637,6 @@
           <t>万磊市场部</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>186-8825-1404, 4000-147-187</t>
@@ -4864,7 +4777,6 @@
           <t>+86-13802465791</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>广东省佛山市顺德区均安镇智安北路12号 (No.12 Zhi'an North Road, Jun'an, Shunde, Foshan, Guangdong, China)</t>
@@ -4872,7 +4784,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -4890,7 +4802,6 @@
           <t>浙江雅柔装饰材料有限公司 (Zhejiang Yarou Decoration Material Co., Ltd.)</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>sale01@yarouwallpaper.com.cn</t>
@@ -4936,13 +4847,11 @@
           <t>戴艳辉</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>18830173388</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>石家庄市正定县曙光路49号东标和聚居</t>
@@ -4950,7 +4859,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5073,8 +4982,6 @@
           <t>+8618901960431</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -5110,7 +5017,6 @@
           <t>13233648687</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>298, Huobei Road, Fuxing Economic Development Zone, Fuxing District, Handan City, Hebei Province</t>
@@ -5136,7 +5042,6 @@
           <t>Foshan Cofesu Sanitary Ware Co., Ltd.</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>sales@cofesu.com</t>
@@ -5192,7 +5097,6 @@
           <t>+86-156-2562-1155</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>Jieyang City, Guangdong Province Jiedong Longwei high-tech Zone industrial Park</t>
@@ -5200,7 +5104,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5233,7 +5137,6 @@
           <t>+86 132 8810 6615</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>Jieyang jiedong district industrial park pandong southeast river science and technology avenue.</t>
@@ -5274,7 +5177,6 @@
           <t>+86 13823419116 / 0758-8565117</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>广东省肇庆市高要区金利镇圩镇社区金灿北路3号 (No. 3 Jinchan North Road, Xuzhen Community, Jinli Town, Gaoyao District, Zhaoqing City, Guangdong China)</t>
@@ -5327,7 +5229,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5345,18 +5247,14 @@
           <t>明德 (Mingde)</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>www.mingde-china.com</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5536,7 +5434,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Doors &amp; Windows</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -5784,14 +5682,11 @@
           <t>张爱彬 (Zhang Aibin)</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
           <t>+86 18178085851</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
           <t>Building Decoration</t>
@@ -6019,7 +5914,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Building Decoration</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">

</xml_diff>

<commit_message>
CBD: translate contact names + add Buyer labels
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>50.000¥. Moq-1</t>
+          <t>Buyer: 50.000¥. Moq-1</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>50.000¥. Moq-1</t>
+          <t>Buyer: 50.000¥. Moq-1</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>50.000¥. Moq-1</t>
+          <t>Buyer: 50.000¥. Moq-1</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>1000 pcs price 38 USD</t>
+          <t>Buyer: 1000 pcs price 38 USD</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>80$</t>
+          <t>Buyer: 80$</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>500pcs / $100USD for pcs</t>
+          <t>Buyer: 500pcs / $100USD for pcs</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Custom order</t>
+          <t>Buyer: Custom order</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Custom order</t>
+          <t>Buyer: Custom order</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>170 to 335 usd</t>
+          <t>Buyer: 170 to 335 usd</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>100 to up</t>
+          <t>Buyer: 100 to up</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>100 to up usd</t>
+          <t>Buyer: 100 to up usd</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>邹隆鹏</t>
+          <t>邹隆鹏 (Zou Longpeng)</t>
         </is>
       </c>
       <c r="D13" s="3" t="n"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Buyer: Super</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>黎桃桃</t>
+          <t>黎桃桃 (Li Taotao)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Buyer: Super</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>曾燕燕 Elyn</t>
+          <t>曾燕燕 Elyn (Zeng Yanyan Elyn)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Buyer: 50</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>王小忠</t>
+          <t>王小忠 (Wang Xiaozhong)</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Buyer: 100</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>应杨军</t>
+          <t>应杨军 (Ying Yangjun)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Buyer: 100</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>顾鹏</t>
+          <t>顾鹏 (Gu Peng)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Wall sheet , 200 rmb per meter , 2000 mtr,</t>
+          <t>Buyer: Wall sheet , 200 rmb per meter , 2000 mtr,</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Handles , 500 moq , 100 rmb per handle</t>
+          <t>Buyer: Handles , 500 moq , 100 rmb per handle</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Wall sheet and wooden wall sheet , 2000mtr , 150 rmb per mtr</t>
+          <t>Buyer: Wall sheet and wooden wall sheet , 2000mtr , 150 rmb per mtr</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>张丽</t>
+          <t>张丽 (Zhang Li)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Price: 800 – 2600 CNY per unit depending on the model and features. MOQ: 100 units for standard orders and 300 units for</t>
+          <t>Buyer: Price: 800 – 2600 CNY per unit depending on the model and features. MOQ: 100 units for standard orders and 300 units for</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>杨苗</t>
+          <t>杨苗 (Yang Miao)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Price: 1200 – 3500 CNY per unit depending on materials and security specifications. MOQ: 50 units for standard models an</t>
+          <t>Buyer: Price: 1200 – 3500 CNY per unit depending on materials and security specifications. MOQ: 50 units for standard models an</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Price: 1800 – 4500 CNY per unit based on the finish and decorative complexity. MOQ: 30 units for standard designs and 10</t>
+          <t>Buyer: Price: 1800 – 4500 CNY per unit based on the finish and decorative complexity. MOQ: 30 units for standard designs and 10</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>赖华芳</t>
+          <t>赖华芳 (Lai Huafang)</t>
         </is>
       </c>
       <c r="D24" s="2" t="n"/>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Хорошее, 400rmb</t>
+          <t>Buyer: Хорошее, 400rmb</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Clément / 付雄豪</t>
+          <t>Clément / 付雄豪 (Clément / Fu Xionghao)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Хорошее , 1500rmb</t>
+          <t>Buyer: Хорошее , 1500rmb</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>周灿灿</t>
+          <t>周灿灿 (Zhou Cancan)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Нормальное</t>
+          <t>Buyer: Нормальное</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>$55, MOQ100pcs, good</t>
+          <t>Buyer: $55, MOQ100pcs, good</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>陈洁玲 Rowling</t>
+          <t>陈洁玲 Rowling (Rowling Chen Jieling (or Chen Jieling Rowling))</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>1000 yuan 1 square</t>
+          <t>Buyer: 1000 yuan 1 square</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>罗美玲</t>
+          <t>罗美玲 (Luo Meiling)</t>
         </is>
       </c>
       <c r="D29" s="3" t="n"/>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>150 rmb</t>
+          <t>Buyer: 150 rmb</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>570 rmb</t>
+          <t>Buyer: 570 rmb</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>130 super</t>
+          <t>Buyer: 130 super</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>$32, MOQ 300, good</t>
+          <t>Buyer: $32, MOQ 300, good</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>¥3000, MoQ 1pcs, very good</t>
+          <t>Buyer: ¥3000, MoQ 1pcs, very good</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>徐小俊</t>
+          <t>徐小俊 (Xu Xiaojun)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>¥17, Moq 50, good</t>
+          <t>Buyer: ¥17, Moq 50, good</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>黄伟业</t>
+          <t>黄伟业 (Huang Weiye)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>600 RMB Great, very cheap</t>
+          <t>Buyer: 600 RMB Great, very cheap</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>10$</t>
+          <t>Buyer: 10$</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>曾令贵</t>
+          <t>曾令贵 (Zeng Linggui)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>69$</t>
+          <t>Buyer: 69$</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>50-85$</t>
+          <t>Buyer: 50-85$</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>陈卓敏 Ruby</t>
+          <t>陈卓敏 Ruby (Ruby Chen Zhuomin)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>￥1000 good</t>
+          <t>Buyer: ￥1000 good</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Crystal 刘晓艺</t>
+          <t>Crystal 刘晓艺 (Crystal Liu Xiaoyi)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>¥ 500 good</t>
+          <t>Buyer: ¥ 500 good</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>￥ 300 good</t>
+          <t>Buyer: ￥ 300 good</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>300 rmb and more. Good quality and good price. Small quantity</t>
+          <t>Buyer: 300 rmb and more. Good quality and good price. Small quantity</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>王闻浠</t>
+          <t>王闻浠 (Wang Wenxi)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>33$ for 1 pcs. Good quality and quantity</t>
+          <t>Buyer: 33$ for 1 pcs. Good quality and quantity</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Good 👍</t>
+          <t>Buyer: Good 👍</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>Buyer: 5800</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>130 yuan</t>
+          <t>Buyer: 130 yuan</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>20000usd</t>
+          <t>Buyer: 20000usd</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>500yuan</t>
+          <t>Buyer: 500yuan</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>MOQ 100, 47 rnb per piece</t>
+          <t>Buyer: MOQ 100, 47 rnb per piece</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>董华</t>
+          <t>董华 (Dong Hua)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>MOQ 50, 200 rnb per</t>
+          <t>Buyer: MOQ 50, 200 rnb per</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>MOQ 10, 845 per piece</t>
+          <t>Buyer: MOQ 10, 845 per piece</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>1pcs. Start from 60rmb. Novative technology</t>
+          <t>Buyer: 1pcs. Start from 60rmb. Novative technology</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>Buyer: 1410</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>洪美兰</t>
+          <t>洪美兰 (Hong Meilan)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>Buyer: 329</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>Buyer: 229</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>潘禹</t>
+          <t>潘禹 (Pan Yu)</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>Buyer: 680</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>150 yuan, 100, good range of products</t>
+          <t>Buyer: 150 yuan, 100, good range of products</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
+          <t>Buyer: Set of furniture is very good quality, I like the company has also a showroom in Guangzhou</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Winni 何玲玲</t>
+          <t>Winni 何玲玲 (Winni He Lingling)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
+          <t>Buyer: The price starts from three thousand yuan, the consultant showed all the functionality and provided a catalogue</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
+          <t>Buyer: 167 юаней , 500 штук минималка . Продукт хороший но у них свое приложение , не работают с Туя и Яндекс Алисой . Будет пр</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>王鹏</t>
+          <t>王鹏 (Wang Peng)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
+          <t>Buyer: 20000 юаней . Качественный продукт, есть свое приложение. Но цена значительно завышена для подобного рода сегмента.</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>劉奕紫 Cathy</t>
+          <t>劉奕紫 Cathy (Cathy Liu Yizi)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
+          <t>Buyer: От одного Саунд Бокса. Стоимость 5000$. Есть возможность при увеличении количества заказа, получить скидку. Очень аккура</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Buyer: 100</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
+          <t>Buyer: MOQ 5 pcs, I got sample price for 2400usd. They have a very innovative product and very trendy. Their service is very go</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
+          <t>Buyer: MOQ 3 for custom made. 800usd. Different sizes different prices. Very affordable and good designs.</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>Buyer: 600</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>0.6 usd/m2</t>
+          <t>Buyer: 0.6 usd/m2</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>王虎旗</t>
+          <t>王虎旗 (Wang Huqi)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Under negotiation, great opportunities</t>
+          <t>Buyer: Under negotiation, great opportunities</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>1-5 usd/l</t>
+          <t>Buyer: 1-5 usd/l</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>6000RMB</t>
+          <t>Buyer: 6000RMB</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>2000RMB&amp;gt;</t>
+          <t>Buyer: 2000RMB&amp;gt;</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>MOQ - 5000 and price - 7000 dollars</t>
+          <t>Buyer: MOQ - 5000 and price - 7000 dollars</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>The price cheap, merchant very friendly</t>
+          <t>Buyer: The price cheap, merchant very friendly</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>The price more cheaper, good quality</t>
+          <t>Buyer: The price more cheaper, good quality</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>严金霞</t>
+          <t>严金霞 (Yan Jinxia)</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Good merchant, perfect products</t>
+          <t>Buyer: Good merchant, perfect products</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>叶小龙/Dustin Ye</t>
+          <t>叶小龙/Dustin Ye (Ye Xiaolong/Dustin Ye)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
+          <t>Buyer: 160 RMB/ pcs The prices are attractive and he wants me to represent their products in my country.</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>15 RMB the product is interesting</t>
+          <t>Buyer: 15 RMB the product is interesting</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>吴仁余</t>
+          <t>吴仁余 (Wu Renyu)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>nearly $15,000 for this production line</t>
+          <t>Buyer: nearly $15,000 for this production line</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>Buyer: 149</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>袁佳磊</t>
+          <t>袁佳磊 (Yuan Jialei)</t>
         </is>
       </c>
       <c r="D80" s="2" t="n"/>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>Buyer: 749</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>5000 USD</t>
+          <t>Buyer: 5000 USD</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
+          <t>Buyer: Smart home system 2000 RMB. They have showed us how the smart home system works. That’s amazing!</t>
         </is>
       </c>
     </row>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>249 RMB. They have fully described their products.</t>
+          <t>Buyer: 249 RMB. They have fully described their products.</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>6000RMB，积极，详细地告诉了一切</t>
+          <t>Buyer: 6000RMB，积极，详细地告诉了一切</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>颜加伟</t>
+          <t>颜加伟 (Yan Jiawei)</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>400rmb /m2 good meeting</t>
+          <t>Buyer: 400rmb /m2 good meeting</t>
         </is>
       </c>
     </row>
@@ -4032,7 +4032,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>高学梅</t>
+          <t>高学梅 (Gao Xuemei)</t>
         </is>
       </c>
       <c r="D86" s="2" t="n"/>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>350 rmb/m2</t>
+          <t>Buyer: 350 rmb/m2</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
+          <t>Buyer: 194 / MOQ 1 Was surprised of price, low price for this beautiful staff</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>20 / MOQ 100 Nice worker answered all questions</t>
+          <t>Buyer: 20 / MOQ 100 Nice worker answered all questions</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>80 rmb for 230 meter</t>
+          <t>Buyer: 80 rmb for 230 meter</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>王冠</t>
+          <t>王冠 (Wang Guan)</t>
         </is>
       </c>
       <c r="D90" s="2" t="n"/>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>1560 rmb for whole item</t>
+          <t>Buyer: 1560 rmb for whole item</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>4600 rmb</t>
+          <t>Buyer: 4600 rmb</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>朱支群</t>
+          <t>朱支群 (Zhu Zhiqun)</t>
         </is>
       </c>
       <c r="D92" s="2" t="n"/>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>250¥/м3</t>
+          <t>Buyer: 250¥/м3</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4353,7 @@
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>4500¥</t>
+          <t>Buyer: 4500¥</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>300¥ 300pcs</t>
+          <t>Buyer: 300¥ 300pcs</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>50¥ 1000pcs</t>
+          <t>Buyer: 50¥ 1000pcs</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Amy Liu 刘建美</t>
+          <t>Amy Liu 刘建美 (Amy Liu / Liu Jianmei)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>500$ 100psc</t>
+          <t>Buyer: 500$ 100psc</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>胡光辉</t>
+          <t>胡光辉 (Hu Guanghui)</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>980y/m2, moq 1000p, like doors with Mosquito netting</t>
+          <t>Buyer: 980y/m2, moq 1000p, like doors with Mosquito netting</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>陈可樑</t>
+          <t>陈可樑 (Chen Keliang)</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>1000-2000p, 1.7-7$, good beautiful doors handless</t>
+          <t>Buyer: 1000-2000p, 1.7-7$, good beautiful doors handless</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>徐云霞</t>
+          <t>徐云霞 (Xu Yunxia)</t>
         </is>
       </c>
       <c r="D99" s="3" t="n"/>
@@ -4607,7 +4607,7 @@
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>100 RMB per sample. The taste is very good</t>
+          <t>Buyer: 100 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>150 RMB per sample. The taste is very good</t>
+          <t>Buyer: 150 RMB per sample. The taste is very good</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea.</t>
+          <t>Buyer: They have tea perfume bar, which was amazing, moreover, i also love their snacks idea with tea.</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>Buyer: I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>Buyer: I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>万磊市场部</t>
+          <t>万磊市场部 (Wan Lei - Marketing Department)</t>
         </is>
       </c>
       <c r="D104" s="2" t="n"/>
@@ -4804,7 +4804,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>I will explore their catalog and website, choose products, then'll make an inquire.</t>
+          <t>Buyer: I will explore their catalog and website, choose products, then'll make an inquire.</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4849,7 @@
       </c>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>Buyer: 1100</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>Buyer: 1050</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>胡沛能 / Oliver Hu</t>
+          <t>胡沛能 / Oliver Hu (Hu Peineng / Oliver Hu)</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="I107" s="3" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>Buyer: 550</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
+          <t>Buyer: 14 RMB per sheet, MOQ is 1000 sheets. The company was agreed to provide shipping services.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>戴艳辉</t>
+          <t>戴艳辉 (Dai Yanhui)</t>
         </is>
       </c>
       <c r="D109" s="3" t="n"/>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
+          <t>Buyer: 0.35 RMB, MOQ is 1000 pieces. Secure packaging material manufactured by this company is good quality</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Melina 王玲</t>
+          <t>Melina 王玲 (Melina Wang Ling)</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>Buyer: 20</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="I111" s="3" t="inlineStr">
         <is>
-          <t>9$</t>
+          <t>Buyer: 9$</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>13.25$</t>
+          <t>Buyer: 13.25$</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="I113" s="3" t="inlineStr">
         <is>
-          <t>8.83$</t>
+          <t>Buyer: 8.83$</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>30 PCs, 420 RMB, need check quality</t>
+          <t>Buyer: 30 PCs, 420 RMB, need check quality</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="I115" s="3" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>Buyer: 10000</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>Buyer: 10000</t>
         </is>
       </c>
     </row>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>邓美君 Jessica</t>
+          <t>邓美君 Jessica (Jessica Deng Meijun)</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="I117" s="3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Buyer: 100</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>Depend on item</t>
+          <t>Buyer: Depend on item</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="I119" s="3" t="inlineStr">
         <is>
-          <t>Depend of quantity</t>
+          <t>Buyer: Depend of quantity</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>刘婉莹 Carol Liu</t>
+          <t>刘婉莹 Carol Liu (Carol Liu Wanying)</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>100/square meter</t>
+          <t>Buyer: 100/square meter</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Jimmy 黄锦民</t>
+          <t>Jimmy 黄锦民 (Jimmy Huang Jinmin)</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="I121" s="3" t="inlineStr">
         <is>
-          <t>RMB 15705 MOQ5; pleasant impression</t>
+          <t>Buyer: RMB 15705 MOQ5; pleasant impression</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>MOQ5 25799 RMB</t>
+          <t>Buyer: MOQ5 25799 RMB</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="I123" s="3" t="inlineStr">
         <is>
-          <t>RMB 19479; MOQ 1</t>
+          <t>Buyer: RMB 19479; MOQ 1</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>Buyer: 1000</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>Buyer: 1000</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>伍乐彤</t>
+          <t>伍乐彤 (Wu Letong (or Ng Lok Tung in Cantonese))</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>2000$, can be customized, very convenient</t>
+          <t>Buyer: 2000$, can be customized, very convenient</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5779,7 @@
       </c>
       <c r="I127" s="3" t="inlineStr">
         <is>
-          <t>38$, very unique</t>
+          <t>Buyer: 38$, very unique</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>2050 rmb, very interesting, convenient to use for pets</t>
+          <t>Buyer: 2050 rmb, very interesting, convenient to use for pets</t>
         </is>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="I129" s="3" t="inlineStr">
         <is>
-          <t>25 rmb, 1 box, like this product</t>
+          <t>Buyer: 25 rmb, 1 box, like this product</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>34 rmb, 1000, normal</t>
+          <t>Buyer: 34 rmb, 1000, normal</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t>40 rmb, 2000, very good</t>
+          <t>Buyer: 40 rmb, 2000, very good</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>周瑶琳</t>
+          <t>周瑶琳 (Zhou Yaolin)</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>1 container 250 rmb</t>
+          <t>Buyer: 1 container 250 rmb</t>
         </is>
       </c>
     </row>
@@ -6037,7 +6037,7 @@
       </c>
       <c r="I133" s="3" t="inlineStr">
         <is>
-          <t>1 container 700 rmb</t>
+          <t>Buyer: 1 container 700 rmb</t>
         </is>
       </c>
     </row>
@@ -6082,7 +6082,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>Цена зависит от обьема, от 3 юаней, расходники</t>
+          <t>Buyer: Цена зависит от обьема, от 3 юаней, расходники</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CBD: translate remaining Chinese chars
</commit_message>
<xml_diff>
--- a/cbd-catalog/cbd_suppliers.xlsx
+++ b/cbd-catalog/cbd_suppliers.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>开平艺和门业有限公司</t>
+          <t>开平艺和门业有限公司 (Kaiping Yihe Door Industry Co., Ltd.)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Crystal Wong 黄健秋</t>
+          <t>Crystal Wong 黄健秋 (Crystal Wong (Huang Jianqiu))</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>邹隆鹏</t>
+          <t>邹隆鹏 (Zou Longpeng)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
@@ -1217,12 +1217,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>广东招材建材科技有限公司</t>
+          <t>广东招材建材科技有限公司 (Guangdong Zhaocai Building Materials Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>黎桃桃</t>
+          <t>黎桃桃 (Li Taotao)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区罗行社区新下村5号厂房</t>
+          <t>广东省佛山市南海区罗行社区新下村5号厂房 (Workshop No. 5, Xinxia Village, Luoxing Community, Nanhai District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>曾燕燕 Elyn</t>
+          <t>曾燕燕 Elyn (Zeng Yanyan (Elyn))</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>杭州南博装饰材料有限公司</t>
+          <t>杭州南博装饰材料有限公司 (Hangzhou Nanbo Decoration Materials Co., Ltd.)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>王小忠</t>
+          <t>王小忠 (Wang Xiaozhong)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1320,7 +1320,7 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>浙江省杭州市临平区运河街道育士路53-1号</t>
+          <t>浙江省杭州市临平区运河街道育士路53-1号 (No. 53-1, Yushi Road, Yunhe Sub-district, Linping District, Hangzhou City, Zhejiang Province)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>台州旭升卫浴股份有限公司</t>
+          <t>台州旭升卫浴股份有限公司 (Taizhou Xusheng Sanitary Ware Co., Ltd.)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>应杨军</t>
+          <t>应杨军 (Ying Yangjun)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>浙江省台州市台州湾新区海虹大道228#</t>
+          <t>浙江省台州市台州湾新区海虹大道228# (No. 228, Haihong Avenue, Taizhou Bay New Area, Taizhou City, Zhejiang Province)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1385,12 +1385,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>NIFO 耐孚</t>
+          <t>NIFO 耐孚 (NIFO Naifu)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>顾鹏</t>
+          <t>顾鹏 (Gu Peng)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Davis Dong 董伟杰</t>
+          <t>Davis Dong 董伟杰 (Davis Dong (Dong Weijie))</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>温州金锏智能锁具有限公司</t>
+          <t>温州金锏智能锁具有限公司 (Wenzhou Jinjian Smart Lock Co., Ltd.)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>张丽</t>
+          <t>张丽 (Zhang Li)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道华盟特色轻工园区1号</t>
+          <t>温州市瓯海区娄桥街道华盟特色轻工园区1号 (No. 1, Huameng Characteristic Light Industry Park, Louqiao Subdistrict, Ouhai District, Wenzhou City)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1553,12 +1553,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>上海世灿国际贸易有限公司</t>
+          <t>上海世灿国际贸易有限公司 (Shanghai Shican International Trade Co., Ltd.)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>杨苗</t>
+          <t>杨苗 (Yang Miao)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>上海市浦东新区商城路889号C3-B06</t>
+          <t>上海市浦东新区商城路889号C3-B06 (C3-B06, No. 889 Shangcheng Road, Pudong New Area, Shanghai)</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>佛山市同路匠人家具有限公司</t>
+          <t>佛山市同路匠人家具有限公司 (Foshan Tonglu Jiangren Furniture Co., Ltd.)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>赖华芳</t>
+          <t>赖华芳 (Lai Huafang)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
@@ -1660,7 +1660,7 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区龙江镇联塑嘉园三路3号9513家具总部</t>
+          <t>广东省佛山市顺德区龙江镇联塑嘉园三路3号9513家具总部 (9513 Furniture Headquarters, No. 3, Liansu Jiayuan 3rd Road, Longjiang Town, Shunde District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>固豪木业 | SUNDIN尚鼎</t>
+          <t>固豪木业 | SUNDIN尚鼎 (Guhao Wood Industry | SUNDIN Shangding)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Clément / 付雄豪</t>
+          <t>Clément / 付雄豪 (Clément / Fu Xionghao)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>周灿灿</t>
+          <t>周灿灿 (Zhou Cancan)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区乐从镇黎湖工业区</t>
+          <t>广东省佛山市顺德区乐从镇黎湖工业区 (Lihu Industrial Zone, Lecong Town, Shunde District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>陈洁玲 Rowling</t>
+          <t>陈洁玲 Rowling (Chen Jieling Rowling)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1902,12 +1902,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>广东省中山名谷屋木门厂</t>
+          <t>广东省中山名谷屋木门厂 (Guangdong Zhongshan Mingguwu Wooden Door Factory)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>罗美玲</t>
+          <t>罗美玲 (Luo Meiling)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
@@ -1919,7 +1919,7 @@
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>广东省中山市小榄镇东升门业生产基地F5B</t>
+          <t>广东省中山市小榄镇东升门业生产基地F5B (F5B, Dongsheng Door Industry Production Base, Xiaolan Town, Zhongshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>超友皮革家居</t>
+          <t>超友皮革家居 (Chaoyou Leather Home Furnishings)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>丰顺县泰雅达实业有限公司</t>
+          <t>丰顺县泰雅达实业有限公司 (Fengshun County Taiyada Industrial Co., Ltd.)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>徐小俊</t>
+          <t>徐小俊 (Xu Xiaojun)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>广东省丰顺县汤坑镇太平北路</t>
+          <t>广东省丰顺县汤坑镇太平北路 (Taiping North Road, Tangkeng Town, Fengshun County, Guangdong Province)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>佛山市悠派家居科技有限公司</t>
+          <t>佛山市悠派家居科技有限公司 (Foshan Youpai Home Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>黄伟业</t>
+          <t>黄伟业 (Huang Weiye)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道古鉴成展路3号</t>
+          <t>广东省佛山市顺德区大良街道古鉴成展路3号 (No. 3 Chengzhan Road, Gujian, Daliang Subdistrict, Shunde District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区郑陆镇工业集中区</t>
+          <t>江苏省常州市天宁区郑陆镇工业集中区 (Industrial Concentration Zone, Zhenglu Town, Tianning District, Changzhou City, Jiangsu Province)</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>曾令贵</t>
+          <t>曾令贵 (Zeng Linggui)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>福建省漳州市长泰区兴泰工业园区台湾工业园锦都路191号</t>
+          <t>福建省漳州市长泰区兴泰工业园区台湾工业园锦都路191号 (No. 191 Jindu Road, Taiwan Industrial Park, Xingtai Industrial Park, Changtai District, Zhangzhou City, Fujian Province)</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2345,12 +2345,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>杭州班昇</t>
+          <t>杭州班昇 (Hangzhou Bansheng)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>陈卓敏 Ruby</t>
+          <t>陈卓敏 Ruby (Ruby Chen Zhuomin)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Crystal 刘晓艺</t>
+          <t>Crystal 刘晓艺 (Crystal Liu Xiaoyi)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>江门市新阳刚智能科技有限公司</t>
+          <t>江门市新阳刚智能科技有限公司 (Jiangmen Xinyanggang Intelligent Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr"/>
@@ -2485,7 +2485,7 @@
       <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>广东省江门市新会区大泽镇万洋众创城38-1号</t>
+          <t>广东省江门市新会区大泽镇万洋众创城38-1号 (No. 38-1, Wanyang Zhongchuang City, Daze Town, Xinhui District, Jiangmen City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
@@ -2505,12 +2505,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>河南蓝健陶瓷有限公司</t>
+          <t>河南蓝健陶瓷有限公司 (Henan Lanjian Ceramics Co., Ltd.)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>王闻浠</t>
+          <t>王闻浠 (Wang Wenxi)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>河南省长葛市石固镇梁庄工业园区</t>
+          <t>河南省长葛市石固镇梁庄工业园区 (Liangzhuang Industrial Park, Shigu Town, Changge City, Henan Province)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>三强地毯</t>
+          <t>三强地毯 (Sanqiang Carpet)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
@@ -2841,12 +2841,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>盐城格子匠家居有限公司</t>
+          <t>盐城格子匠家居有限公司 (Yancheng Gezijiang Home Furnishing Co., Ltd.)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>董华</t>
+          <t>董华 (Dong Hua)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2862,7 +2862,7 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>江苏省盐城市亭湖区青墩头灶工业园全创路十号</t>
+          <t>江苏省盐城市亭湖区青墩头灶工业园全创路十号 (No. 10, Quanchuang Road, Qingdun Touzao Industrial Park, Tinghu District, Yancheng City, Jiangsu Province)</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Jasmine Guan 管敏秀</t>
+          <t>Jasmine Guan 管敏秀 (Jasmine Guan (Guan Minxiu))</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2927,12 +2927,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>利亚德光电股份有限公司 Leyard Optoelectronic Co., Ltd.</t>
+          <t>利亚德光电股份有限公司 Leyard Optoelectronic Co., Ltd. (Leyard Optoelectronic Co., Ltd.)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>金厚强 Jin Houqiang</t>
+          <t>金厚强 Jin Houqiang (Jin Houqiang)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>北京市海淀区颐和园北正红旗西街9号 / 深圳市龙华区观澜街道君子布社区观和路6号深圳利亚德微LED南方产业园A栋</t>
+          <t>北京市海淀区颐和园北正红旗西街9号 / 深圳市龙华区观澜街道君子布社区观和路6号深圳利亚德微LED南方产业园A栋 (No. 9, Zhenghongqi West Street, North of Summer Palace, Haidian District, Beijing / Block A, Shenzhen Leyard Micro LED Southern Industrial Park, No. 6, Guanhe Road, Junzibu Community, Guanlan Street, Longhua District, Shenzhen)</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3047,12 +3047,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>JNOD 基诺德</t>
+          <t>JNOD 基诺德 (JNOD)</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>周信朋 Joe Zhou</t>
+          <t>周信朋 Joe Zhou (Joe Zhou (Zhou Xinpeng))</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3088,12 +3088,12 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>广州传祺时代智能科技有限公司</t>
+          <t>广州传祺时代智能科技有限公司 (Guangzhou Chuanqi Times Intelligent Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>洪美兰</t>
+          <t>洪美兰 (Hong Meilan)</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>广州市黄埔区云埔工业区观达路20号密博科技园</t>
+          <t>广州市黄埔区云埔工业区观达路20号密博科技园 (Mibo Science Park, No. 20, Guanda Road, Yunpu Industrial Zone, Huangpu District, Guangzhou)</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>潘禹</t>
+          <t>潘禹 (Pan Yu)</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr"/>
@@ -3191,7 +3191,7 @@
       <c r="F69" s="3" t="inlineStr"/>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>广东省惠州市惠城区演达大道19号国安居6楼</t>
+          <t>广东省惠州市惠城区演达大道19号国安居6楼 (6th Floor, Guo'anju, No. 19 Yanda Avenue, Huicheng District, Huizhou City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Winni 何玲玲</t>
+          <t>Winni 何玲玲 (Winni He Lingling)</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>视威电子科技（上海）有限公司</t>
+          <t>视威电子科技（上海）有限公司 (Shiwei Electronic Technology (Shanghai) Co., Ltd. (or SWIT Electronics Technology (Shanghai) Co., Ltd.))</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr"/>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>上海市闵行区新骏环路188号11号楼A座518室</t>
+          <t>上海市闵行区新骏环路188号11号楼A座518室 (Room 518, Block A, Building 11, No. 188 Xinjunhuan Road, Minhang District, Shanghai)</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3408,12 +3408,12 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>爱舒床垫集团有限公司</t>
+          <t>爱舒床垫集团有限公司 (Aishu Mattress Group Co., Ltd.)</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>王鹏</t>
+          <t>王鹏 (Wang Peng)</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>劉奕紫 Cathy</t>
+          <t>劉奕紫 Cathy (Liu Yizi Cathy)</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -3811,12 +3811,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>河南威兰得建筑科技有限公司</t>
+          <t>河南威兰得建筑科技有限公司 (Henan Weilande Building Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>王虎旗</t>
+          <t>王虎旗 (Huqi Wang)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>河南省郑州市曲梁工业园188号</t>
+          <t>河南省郑州市曲梁工业园188号 (No. 188, Quliang Industrial Park, Zhengzhou City, Henan Province)</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>江门市新会区致恒科技材料有限公司</t>
+          <t>江门市新会区致恒科技材料有限公司 (Jiangmen City Xinhui District Zhiheng Technology Materials Co., Ltd.)</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -3873,7 +3873,7 @@
       <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>广东省江门市蓬江区迎宾大道西23号之129</t>
+          <t>广东省江门市蓬江区迎宾大道西23号之129 (No. 23-129, West Yingbin Avenue, Pengjiang District, Jiangmen City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>双龙智科</t>
+          <t>双龙智科 (Shuanglong Zhike (or Shuanglong Intelligent Technology))</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr"/>
@@ -4063,7 +4063,7 @@
       <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>江苏省太仓市双凤镇陆江路1号</t>
+          <t>江苏省太仓市双凤镇陆江路1号 (No. 1, Lujiang Road, Shuangfeng Town, Taicang City, Jiangsu Province)</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
@@ -4190,7 +4190,7 @@
       <c r="F96" s="2" t="inlineStr"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>中国广东省佛山市南海区里水镇大步工业区13号 (No. 13, Dabu Industrial Zone, Lishui Town, Nanhai District, Foshan City, Guangdong Province, China)</t>
+          <t>中国广东省佛山市南海区里水镇 (Lishui Town, Nanhai District, Foshan City, Guangdong Province)大步工业区13号 (No. 13, Dabu Industrial Zone, Lishui Town, Nanhai District, Foshan City, Guangdong Province, China)</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -4251,12 +4251,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>广州蒙娜丽莎控股集团有限公司, 广州蒙娜丽莎卫浴股份有限公司</t>
+          <t>广州蒙娜丽莎控股集团有限公司, 广州蒙娜丽莎卫浴股份有限公司 (Guangzhou Mona Lisa Holding Group Co., Ltd., Guangzhou Mona Lisa Sanitary Ware Co., Ltd.)</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>严金霞</t>
+          <t>严金霞 (Jinxia Yan)</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇港头工业区4号</t>
+          <t>广州市花都区花东镇港头工业区4号 (No. 4, Gangtou Industrial Zone, Huadong Town, Huadu District, Guangzhou City)</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>叶小龙/Dustin Ye</t>
+          <t>叶小龙/Dustin Ye (Xiaolong Ye/Dustin Ye)</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -4386,12 +4386,12 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>浙江瑞鑫环保设备有限公司</t>
+          <t>浙江瑞鑫环保设备有限公司 (Zhejiang Ruixin Environmental Protection Equipment Co., Ltd.)</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>吴仁余</t>
+          <t>吴仁余 (Renyu Wu)</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>浙江省金华市婺城区罗店镇北山路精工工业园</t>
+          <t>浙江省金华市婺城区罗店镇北山路精工工业园 (Jinggong Industrial Park, Beishan Road, Luodian Town, Wucheng District, Jinhua City, Zhejiang Province)</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
@@ -4476,12 +4476,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>苏州市富尔达科技股份有限公司</t>
+          <t>苏州市富尔达科技股份有限公司 (Suzhou Fuerda Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>袁佳磊</t>
+          <t>袁佳磊 (Jialei Yuan)</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr"/>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>江苏省太仓市港区临江路1号</t>
+          <t>江苏省太仓市港区临江路1号 (No. 1, Linjiang Road, Port Area, Taicang City, Jiangsu Province)</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>双龙中科</t>
+          <t>双龙中科 (Shuanglong Zhongke)</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr"/>
@@ -4575,7 +4575,7 @@
       <c r="F105" s="3" t="inlineStr"/>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>江苏省太仓市双凤镇陆江路1号</t>
+          <t>江苏省太仓市双凤镇陆江路1号 (No. 1, Lujiang Road, Shuangfeng Town, Taicang City, Jiangsu Province)</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>深圳市家为安智能科技有限公司</t>
+          <t>深圳市家为安智能科技有限公司 (Shenzhen Jiaweian Intelligent Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr"/>
@@ -4608,7 +4608,7 @@
       <c r="F106" s="2" t="inlineStr"/>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区里水镇</t>
+          <t>广东省佛山市南海区里水镇 (Lishui Town, Nanhai District, Foshan City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>广州市优品声学科技有限公司</t>
+          <t>广州市优品声学科技有限公司 (Guangzhou Youpin Acoustic Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr"/>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>广东省广州市番禺区南村镇南村西路138号德意创意园二层</t>
+          <t>广东省广州市番禺区南村镇南村西路138号德意创意园二层 (2nd Floor, Deyi Creative Park, No. 138 Nancun West Road, Nancun Town, Panyu District, Guangzhou City, Guangdong Province)</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr">
@@ -4690,12 +4690,12 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>贵州佑远木业有限公司</t>
+          <t>贵州佑远木业有限公司 (Guizhou Youyuan Wood Industry Co., Ltd.)</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>颜加伟</t>
+          <t>颜加伟 (Jiawei Yan)</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>高学梅</t>
+          <t>高学梅 (Xuemei Gao)</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr"/>
@@ -4899,7 +4899,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>江西荣科新型材料有限公司 / JIANGXI RONGKE NEW BUILDING MATERIALS CO., LTD.</t>
+          <t>江西荣科新型材料有限公司 / JIANGXI RONGKE NEW BUILDING MATERIALS CO., LTD. (Jiangxi Rongke New Building Materials Co., Ltd.)</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>王冠</t>
+          <t>王冠 (Guan Wang)</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr"/>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="G115" s="3" t="inlineStr">
         <is>
-          <t>展厅：佛山市禅城区季华西路68号中国陶瓷产业总部基地东区C03座；工厂：佛山市南海区狮山谭边工业二区</t>
+          <t>展厅：佛山市禅城区季华西路68号中国陶瓷产业总部基地东区C03座；工厂：佛山市南海区狮山谭边工业二区 (Showroom: Block C03, East Area, China Ceramics Headquarters, No. 68 Jihua West Road, Chancheng District, Foshan City; Factory: Tanbian No. 2 Industrial Zone, Shishan Town, Nanhai District, Foshan City)</t>
         </is>
       </c>
       <c r="H115" s="3" t="inlineStr">
@@ -5096,12 +5096,12 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>江西瑞京鸿兴实业有限公司</t>
+          <t>江西瑞京鸿兴实业有限公司 (Jiangxi Ruijing Hongxing Industrial Co., Ltd.)</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>朱支群</t>
+          <t>朱支群 (Zhiqun Zhu)</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr"/>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>江西省瑞金市经济开发区创业一路东侧</t>
+          <t>江西省瑞金市经济开发区创业一路东侧 (East Side of Chuangye 1st Road, Economic Development Zone, Ruijin City, Jiangxi Province)</t>
         </is>
       </c>
       <c r="H119" s="3" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Amy Liu 刘建美</t>
+          <t>Amy Liu 刘建美 (Amy Liu (Jianmei Liu))</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -5358,12 +5358,12 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>佛山市旌晨铝门窗有限公司</t>
+          <t>佛山市旌晨铝门窗有限公司 (Foshan Jingchen Aluminum Doors and Windows Co., Ltd.)</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>胡光辉</t>
+          <t>胡光辉 (Hu Guanghui)</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -5379,7 +5379,7 @@
       <c r="F125" s="3" t="inlineStr"/>
       <c r="G125" s="3" t="inlineStr">
         <is>
-          <t>佛山狮山镇谭边工业区崩岗头路四号之一</t>
+          <t>佛山狮山镇谭边工业区崩岗头路四号之一 (No. 4-1 Benggangtou Road, Tanbian Industrial Zone, Shishan Town, Foshan City)</t>
         </is>
       </c>
       <c r="H125" s="3" t="inlineStr">
@@ -5399,12 +5399,12 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>佛山市乾泽科技有限公司</t>
+          <t>佛山市乾泽科技有限公司 (Foshan Qianze Technology Co., Ltd.)</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>陈可樑</t>
+          <t>陈可樑 (Chen Keliang)</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>广东省佛山市三水区云东海街道宝盛路2号1座三层（合和建筑五金园区北门）</t>
+          <t>广东省佛山市三水区云东海街道宝盛路2号1座三层（合和建筑五金园区北门） (3rd Floor, Block 1, No. 2 Baosheng Road, Yundonghai Sub-district, Sanshui District, Foshan City, Guangdong Province (North Gate of Hehe Architectural Hardware Park))</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>PTAT | 帕兰蒂诺</t>
+          <t>PTAT | 帕兰蒂诺 (PTAT | Palatino)</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -5563,12 +5563,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>万磊建筑涂料有限公司</t>
+          <t>万磊建筑涂料有限公司 (Wanlei Architectural Coatings Co., Ltd.)</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>万磊市场部</t>
+          <t>万磊市场部 (Wan Lei, Marketing Department)</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>总部：广东省佛山市南海区松岗万石工业区；分厂：广西省贵港市覃塘区产业园甘化园区</t>
+          <t>总部：广东省佛山市南海区松岗万石工业区；分厂：广西省贵港市覃塘区产业园甘化园区 (Headquarters: Wanshi Industrial Zone, Songgang, Nanhai District, Foshan City, Guangdong Province; Branch Factory: Ganhua Zone, Industrial Park, Qintang District, Guigang City, Guangxi Province)</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -5851,12 +5851,12 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>淄博永顺装饰材料有限公司</t>
+          <t>淄博永顺装饰材料有限公司 (Zibo Yongshun Decorative Materials Co., Ltd.)</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>戴艳辉</t>
+          <t>戴艳辉 (Dai Yanhui)</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr"/>
@@ -5868,7 +5868,7 @@
       <c r="F138" s="2" t="inlineStr"/>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>石家庄市正定县曙光路49号东标和聚居</t>
+          <t>石家庄市正定县曙光路49号东标和聚居 (Dongbiao Hejuju, No. 49 Shuguang Road, Zhengding County, Shijiazhuang City)</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Melina 王玲</t>
+          <t>Melina 王玲 (Melina Wang Ling)</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>邓美君 Jessica</t>
+          <t>邓美君 Jessica (Jessica Deng Meijun)</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>刘婉莹 Carol Liu</t>
+          <t>刘婉莹 Carol Liu (Carol Liu Wanying)</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>Jimmy 黄锦民</t>
+          <t>Jimmy 黄锦民 (Jimmy Huang Jinmin)</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>伍乐彤</t>
+          <t>伍乐彤 (Wu Letong)</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="G157" s="3" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇港头工业区4号</t>
+          <t>广州市花都区花东镇港头工业区4号 (No. 4, Gangtou Industrial Zone, Huadong Town, Huadu District, Guangzhou City)</t>
         </is>
       </c>
       <c r="H157" s="3" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>河北省泊头市寺门村镇后牛屯</t>
+          <t>河北省泊头市寺门村镇后牛屯 (Houniutun, Simencun Town, Botou City, Hebei Province)</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
@@ -6900,12 +6900,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>浙江安吉双虎竹木业有限公司 / 安吉诺迪新材料有限公司</t>
+          <t>浙江安吉双虎竹木业有限公司 / 安吉诺迪新材料有限公司 (Zhejiang Anji Shuanghu Bamboo &amp; Wood Industry Co., Ltd. / Anji Nuodi New Material Co., Ltd.)</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>周瑶琳</t>
+          <t>周瑶琳 (Zhou Yaolin)</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -6925,7 +6925,7 @@
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
-          <t>浙江省湖州市安吉县孝丰镇大竹村</t>
+          <t>浙江省湖州市安吉县孝丰镇大竹村 (Dazhu Village, Xiaofeng Town, Anji County, Huzhou City, Zhejiang Province)</t>
         </is>
       </c>
       <c r="H163" s="3" t="inlineStr">
@@ -6945,12 +6945,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>宏宇集团 HONGYU GROUP</t>
+          <t>宏宇集团 HONGYU GROUP (Hongyu Group HONGYU GROUP)</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Melina 王玲</t>
+          <t>Melina 王玲 (Melina Wang Ling)</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">

</xml_diff>